<commit_message>
Apple top 100 ingelezen: vierkante covers, themas en ranglijst
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -434,6 +434,11 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -462,6 +467,31 @@
           <t>website</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>thema</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>omschrijving</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>omschrijving_lang</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>apple_id</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>apple_rang</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -479,6 +509,23 @@
       </c>
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Comedy</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Bas Louissen, Chris Bergstrom en Puck van den Hoogen maken elke ochtend een korte podcast over het nieuws waar verder niemand het over heeft.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Hagelslag is een dagelijkse ochtendpodcast van Bas Louissen en Chris Bergstrom, bekend van Man Man Man, samen met Puck van den Hoogen. Geen zware analyses, maar een luchtig magazine vol kleine en bizarre nieuwsberichten. In de theaterversie brengen ze diezelfde chaos en gezelligheid naar de zaal, in een avondvullend programma met vrije stoelkeuze.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -491,11 +538,34 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>https://static.wixstatic.com/media/a81d58_16229e6dcef744f5a41b54d958a2af8d~mv2.jpg</t>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts211/v4/53/40/ed/5340ede4-d2b5-6915-eb4b-00598083ea78/mza_11107074210746792588.jpg/600x600bb.png</t>
         </is>
       </c>
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>True crime</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Misdaadjournalist Wouter Laumans en strafrechtadvocaat Christian Flokstra pluizen elke week een strafzaak uit, van dossier tot vonnis.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Napleiten is een van de best beluisterde true-crimepodcasts van Nederland en werd bekroond als beste podcast van het land. Journalist Wouter Laumans en advocaat Christian Flokstra kijken achter de krantenkoppen: wat speelde er werkelijk in een zaak, en waarom besliste de rechter zoals hij besliste. In de theatertour nemen ze per regio een nieuwe zaak onder de loep, samen met gasten, met ruimte voor vragen uit de zaal. De show wordt geproduceerd door Corti Media Live in samenwerking met BNR.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>1591011702</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -513,6 +583,23 @@
       </c>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Kind &amp; gezin</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Kluun en Yvanka van der Zwaan bespreken alles wat ouders van pubers tegenkomen, van dichtslaande deuren tot schoolstress.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>In ruim honderd afleveringen van Help, ik heb een puber! praten schrijver Kluun en orthopedagoog Yvanka van der Zwaan met experts en met pubers zelf over opvoeden in de puberteit. In de theatershow Best of komen de meest gestelde vragen en de meest herkenbare onderwerpen uit de podcast samen in een avond met veel ruimte voor gesprek met de zaal.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -520,16 +607,39 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Boekestijn &amp; De Wijk</t>
+          <t>Boekestijn en De Wijk</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>https://static.wixstatic.com/media/a81d58_66842450237c4026b22e8e3fb371f5fa~mv2.jpg/v1/fill/w_980,h_1386,al_c,q_85,usm_0.66_1.00_0.01,enc_avif,quality_auto/A4_BDW_26.jpg</t>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts112/v4/7d/f0/e7/7df0e76d-b705-cf2a-94c6-a10ff291497e/mza_16718794314625024290.jpg/600x600bb.png</t>
         </is>
       </c>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Nieuws &amp; politiek</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Arend Jan Boekestijn en Rob de Wijk ontleden voor BNR wekelijks de wereldpolitiek: oorlog, diplomatie en verschuivende machtsverhoudingen.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Boekestijn en De Wijk is de geopolitieke podcast van BNR Nieuwsradio, waarin historicus en oud-politicus Arend Jan Boekestijn en veiligheidsdeskundige Rob de Wijk de wereld van vandaag duiden. In de eindejaarsshow blikken ze samen met host Hugo Reitsma terug op het afgelopen jaar en vooruit op wat komt. De voorstelling is geregisseerd door Peter de Baan en wordt geproduceerd door Corti Media Live, met BNR als partner.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>1076289388</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Paginabouwer: agenda, catalogus, toplijst, pagina per podcast, favorieten, sitemap
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -828,7 +828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -880,6 +880,16 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>laatst_gecheckt</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>prijs_vanaf</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>tijd_bron</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aanvangstijden en prijzen van 41 theaterpaginas, alle 27 zalen op de kaart, uitverkocht zichtbaar, CLAUDE.md bijgewerkt
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -928,6 +928,14 @@
           <t>2026-08-30</t>
         </is>
       </c>
+      <c r="I2" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>https://ticket.tivolivredenburg.nl/nl/buyingflow/tickets/60072/122508</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -941,7 +949,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-26 20:00</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -962,6 +970,14 @@
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>https://stadsschouwburghaarlem.nl/en/agenda/theatercollege-napleiten-live-wouter-laumans-en-christian-flokstra</t>
         </is>
       </c>
     </row>
@@ -977,7 +993,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-29 20:00</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -998,6 +1014,14 @@
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.musisenstadstheater.nl/nl/agenda/wouter-laumans-christian-flokstra-napleiten-live-2026/10204</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1037,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-08 20:00</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1034,6 +1058,14 @@
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.plt.nl/programma/napleiten-live/08-10-2026-20-00</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1081,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-13 20:15</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1070,6 +1102,14 @@
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>https://meervaart.nl/agenda/napleiten-live</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1125,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-22 20:00</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1106,6 +1146,14 @@
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>https://luxortheater.nl/agenda/napleiten-live-56647</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1169,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-11-04</t>
+          <t>2026-11-04 20:00</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1142,6 +1190,14 @@
       <c r="H8" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.schouwburghengelo.nl/napleiten-live-wouter-laumans-en-christian-flokstra/04-11-2026-20-00</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1213,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-11-12 20:15</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1178,6 +1234,14 @@
       <c r="H9" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kampanje.nl/voorstellingen/napleiten-live-sp5r</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1257,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-11-17</t>
+          <t>2026-11-17 20:15</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1214,6 +1278,14 @@
       <c r="H10" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>https://leidseschouwburg-stadsgehoorzaal.nl/voorstelling/wouter-laumans-christian-flokstra-e-a-napleiten-live/</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1301,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-11-26</t>
+          <t>2026-11-26 20:15</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1250,6 +1322,14 @@
       <c r="H11" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>https://kunstlinie.nl/programma/napleiten-live/</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1345,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2027-01-08</t>
+          <t>2027-01-08 20:00</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1286,6 +1366,14 @@
       <c r="H12" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.parktheater.nl/programma/napleiten-live-mjbw</t>
         </is>
       </c>
     </row>
@@ -1324,6 +1412,8 @@
           <t>2026-08-30</t>
         </is>
       </c>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1337,7 +1427,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2027-02-04</t>
+          <t>2027-02-04 20:00</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1358,6 +1448,14 @@
       <c r="H14" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.agnietenhof.nl/agenda/napleiten-live-6sjb</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1471,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2027-02-10</t>
+          <t>2027-02-10 20:00</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1394,6 +1492,14 @@
       <c r="H15" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>https://delamar.nl/voorstellingen/napleiten-live/</t>
         </is>
       </c>
     </row>
@@ -1409,7 +1515,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2027-02-18</t>
+          <t>2027-02-18 20:15</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1430,6 +1536,14 @@
       <c r="H16" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>https://harmonie.nl/agenda/napleiten-live/53059</t>
         </is>
       </c>
     </row>
@@ -1445,7 +1559,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2027-03-04</t>
+          <t>2027-03-04 20:00</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1466,6 +1580,14 @@
       <c r="H17" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.schouwburghengelo.nl/napleiten-live-wouter-laumans-en-christian-flokstra-2/04-03-2027-20-00</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1603,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2027-03-10</t>
+          <t>2027-03-10 20:15</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1502,6 +1624,14 @@
       <c r="H18" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.schouwburgconcertzaaltilburg.nl/nl/agenda/napleiten-live-wouter-laumans-christian-flokstra</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1647,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2027-03-17</t>
+          <t>2027-03-17 20:00</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1538,6 +1668,14 @@
       <c r="H19" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.musisenstadstheater.nl/nl/agenda/wouter-laumans-christian-flokstra-napleiten-live-voorjaar-2027/10205</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1723,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>2027-03-30</t>
+          <t>2027-03-30 20:00</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1606,6 +1744,14 @@
       <c r="H21" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>https://goudseschouwburg.nl/agenda/napleiten-live-10025644/</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1767,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2027-04-07</t>
+          <t>2027-04-07 20:00</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1642,6 +1788,14 @@
       <c r="H22" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amphion.nl/theater/napleiten-live-naar-de-gelijknamige-podcast/</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1811,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2027-04-21</t>
+          <t>2027-04-21 20:00</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1678,6 +1832,14 @@
       <c r="H23" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>https://luxortheater.nl/agenda/napleiten-live-56647</t>
         </is>
       </c>
     </row>
@@ -1693,7 +1855,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2027-05-21</t>
+          <t>2027-05-21 20:00</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1714,6 +1876,14 @@
       <c r="H24" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theateraandeparade.nl/nl/programma/napleiten-live-met-oa-wouter-laumans-christian-flokstra</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1899,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-07 20:15</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1750,6 +1920,14 @@
       <c r="H25" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lievekamp.nl/programma/met-kluun-yvanka-van-der-zwaan-the-best-of-help-ik-heb-een-puber-07-okt-20-15/</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1943,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-28 20:30</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1786,6 +1964,14 @@
       <c r="H26" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>https://delamar.nl/voorstellingen/best-of-help-ik-heb-een-puber-live/</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1987,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-30 20:15</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1822,6 +2008,14 @@
       <c r="H27" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.spotgroningen.nl/programma/kluun-en-yvanka-van-der-zwaan/</t>
         </is>
       </c>
     </row>
@@ -1837,7 +2031,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2026-11-25</t>
+          <t>2026-11-25 20:00</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1858,6 +2052,14 @@
       <c r="H28" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.schouwburgconcertzaaltilburg.nl/nl/agenda/kluun-help-ik-heb-een-puber</t>
         </is>
       </c>
     </row>
@@ -1873,7 +2075,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2026-12-02</t>
+          <t>2026-12-02 20:00</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1894,6 +2096,14 @@
       <c r="H29" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theateraandeparade.nl/nl/programma/the-best-of-help-ik-heb-een-p-kluun</t>
         </is>
       </c>
     </row>
@@ -1909,7 +2119,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>2026-11-03</t>
+          <t>2026-11-03 20:15</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1930,6 +2140,12 @@
       <c r="H30" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="n"/>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theaterdeveste.nl/programma/boekestijn-en-de-wijk-omarmen-de-ondergang-h9ks</t>
         </is>
       </c>
     </row>
@@ -1945,7 +2161,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2026-11-09 20:15</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1966,6 +2182,14 @@
       <c r="H31" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.markantmaashorst.nl/nl/agenda/boekestijn-de-wijk-live-f7k3</t>
         </is>
       </c>
     </row>
@@ -1981,7 +2205,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-11-16 19:30</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2002,6 +2226,14 @@
       <c r="H32" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dekringroosendaal.nl/agenda/boekestijn-de-wijk-live-eindejaars-26-nrz5</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2249,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-11-19 20:00</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -2038,6 +2270,14 @@
       <c r="H33" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.plt.nl/programma/boekestijn-de-wijk-live/19-11-2026-20-00</t>
         </is>
       </c>
     </row>
@@ -2108,6 +2348,8 @@
           <t>2026-08-30</t>
         </is>
       </c>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -2121,7 +2363,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-12-01 20:00</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2142,6 +2384,14 @@
       <c r="H36" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.agnietenhof.nl/agenda/boekestijn-de-wijk-live-8kbs</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2407,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-12-03 20:00</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2178,6 +2428,14 @@
       <c r="H37" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amphion.nl/theater/boekestijn-de-wijk-live-eindejaars-26/</t>
         </is>
       </c>
     </row>
@@ -2193,7 +2451,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>2026-12-08</t>
+          <t>2026-12-08 20:15</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2214,6 +2472,14 @@
       <c r="H38" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>https://leidseschouwburg-stadsgehoorzaal.nl/voorstelling/boekestijn-de-wijk-live-eindejaarsshow-2026/</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2495,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>2026-12-10</t>
+          <t>2026-12-10 20:15</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2250,6 +2516,14 @@
       <c r="H39" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.junushoff.nl/programma/boekestijn-en-de-wijk-skgp</t>
         </is>
       </c>
     </row>
@@ -2265,7 +2539,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>2026-12-12</t>
+          <t>2026-12-12 20:00</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2275,7 +2549,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>in verkoop</t>
+          <t>uitverkocht</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -2286,6 +2560,14 @@
       <c r="H40" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.chasse.nl/nl/programma/boekestijn-de-wijk-live-eindejaars-26-cpbk</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2583,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-12-14 20:00</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2322,6 +2604,14 @@
       <c r="H41" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>https://goudseschouwburg.nl/agenda/boekestijn-de-wijk-live-eindejaars-26-10025643/</t>
         </is>
       </c>
     </row>
@@ -2337,7 +2627,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-12-16 20:15</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2358,6 +2648,14 @@
       <c r="H42" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>https://meervaart.nl/agenda/boekestijn-de-wijk</t>
         </is>
       </c>
     </row>
@@ -2373,7 +2671,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>2026-12-17</t>
+          <t>2026-12-17 20:00</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2394,6 +2692,14 @@
       <c r="H43" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>https://luxortheater.nl/agenda/boekestijn-de-wijk-live-58804</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2715,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>2026-12-21</t>
+          <t>2026-12-21 20:30</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2430,6 +2736,14 @@
       <c r="H44" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.musisenstadstheater.nl/nl/agenda/boekestijn-de-wijk-live-eindejaarsshow-2026/10155</t>
         </is>
       </c>
     </row>
@@ -2445,7 +2759,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>2026-12-22</t>
+          <t>2026-12-22 20:15</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2466,6 +2780,14 @@
       <c r="H45" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.schouwburgconcertzaaltilburg.nl/nl/agenda/boekestijn-de-wijk-live-eindejaars-26</t>
         </is>
       </c>
     </row>
@@ -2568,8 +2890,12 @@
           <t>Noord-Holland</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
+      <c r="E3" s="2" t="n">
+        <v>52.3779947</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>4.625426</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -2720,8 +3046,12 @@
           <t>Noord-Holland</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
+      <c r="E9" s="2" t="n">
+        <v>52.9585736</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>4.7690842</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -2768,8 +3098,12 @@
           <t>Flevoland</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
+      <c r="E11" s="2" t="n">
+        <v>52.3669292</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>5.2191822</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -2790,8 +3124,12 @@
           <t>Noord-Brabant</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
+      <c r="E12" s="2" t="n">
+        <v>51.4288468</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>5.4847037</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -3020,8 +3358,12 @@
           <t>Noord-Brabant</t>
         </is>
       </c>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
+      <c r="E21" s="2" t="n">
+        <v>51.7633501</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>5.5213587</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -3029,7 +3371,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>SPOT Groningen</t>
+          <t>SPOT Stadsschouwburg</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3042,8 +3384,12 @@
           <t>Groningen</t>
         </is>
       </c>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
+      <c r="E22" s="2" t="n">
+        <v>53.2208535</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>6.5720279</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -3064,8 +3410,12 @@
           <t>Zuid-Holland</t>
         </is>
       </c>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
+      <c r="E23" s="2" t="n">
+        <v>52.0084756</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>4.3627946</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -3086,8 +3436,12 @@
           <t>Noord-Brabant</t>
         </is>
       </c>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
+      <c r="E24" s="2" t="n">
+        <v>51.6571579</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>5.6174239</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -3108,8 +3462,12 @@
           <t>Noord-Brabant</t>
         </is>
       </c>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
+      <c r="E25" s="2" t="n">
+        <v>51.5333416</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>4.4586306</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -3130,8 +3488,12 @@
           <t>Limburg</t>
         </is>
       </c>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
+      <c r="E26" s="2" t="n">
+        <v>50.9987922</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>5.8612019</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -3152,8 +3514,12 @@
           <t>Gelderland</t>
         </is>
       </c>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
+      <c r="E27" s="2" t="n">
+        <v>51.9667769</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>5.6614496</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -3161,7 +3527,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Chasse Theater</t>
+          <t>Chassé Theater</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -3174,8 +3540,12 @@
           <t>Noord-Brabant</t>
         </is>
       </c>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
+      <c r="E28" s="2" t="n">
+        <v>51.5874733</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>4.7821816</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fundament voor opschalen: zaalaliassen, inleesroutine zonder dubbelingen, verrijkingsafspraak
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -2802,7 +2802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2811,6 +2811,7 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2844,6 +2845,11 @@
           <t>lon</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>aliassen</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -2870,6 +2876,7 @@
       <c r="F2" s="2" t="n">
         <v>5.1127685</v>
       </c>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -2896,6 +2903,11 @@
       <c r="F3" s="2" t="n">
         <v>4.625426</v>
       </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Stadsschouwburg Haarlem</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -2922,6 +2934,11 @@
       <c r="F4" s="2" t="n">
         <v>5.9137995</v>
       </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Musis Sacrum; Musis en Stadstheater</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -2948,6 +2965,11 @@
       <c r="F5" s="2" t="n">
         <v>5.9727811</v>
       </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Parkstad Limburg Theaters; Theater Heerlen; PLT</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -2974,6 +2996,11 @@
       <c r="F6" s="2" t="n">
         <v>4.8073957</v>
       </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Meervaart Theater; Theater de Meervaart</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -3000,6 +3027,7 @@
       <c r="F7" s="2" t="n">
         <v>4.4911848</v>
       </c>
+      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -3026,6 +3054,11 @@
       <c r="F8" s="2" t="n">
         <v>6.7952206</v>
       </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Schouwburg Hengelo</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -3052,6 +3085,11 @@
       <c r="F9" s="2" t="n">
         <v>4.7690842</v>
       </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Schouwburg De Kampanje; Kampanje</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -3078,6 +3116,11 @@
       <c r="F10" s="2" t="n">
         <v>4.4890446</v>
       </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Leidse Schouwburg; Leidse Schouwburg &amp; Stadsgehoorzaal; Stadsgehoorzaal Leiden</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -3104,6 +3147,7 @@
       <c r="F11" s="2" t="n">
         <v>5.2191822</v>
       </c>
+      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -3130,6 +3174,7 @@
       <c r="F12" s="2" t="n">
         <v>5.4847037</v>
       </c>
+      <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -3156,6 +3201,7 @@
       <c r="F13" s="2" t="n">
         <v>6.0976158</v>
       </c>
+      <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -3182,6 +3228,7 @@
       <c r="F14" s="2" t="n">
         <v>5.436108</v>
       </c>
+      <c r="G14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -3208,6 +3255,7 @@
       <c r="F15" s="2" t="n">
         <v>4.8806878</v>
       </c>
+      <c r="G15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -3234,6 +3282,11 @@
       <c r="F16" s="2" t="n">
         <v>5.7900791</v>
       </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>De Harmonie; Stadsschouwburg de Harmonie</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -3260,6 +3313,11 @@
       <c r="F17" s="2" t="n">
         <v>5.082737</v>
       </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Schouwburg; Concertzaal Tilburg; Schouwburg Tilburg; Concertzaal</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -3286,6 +3344,11 @@
       <c r="F18" s="2" t="n">
         <v>4.7124332</v>
       </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>De Goudse Schouwburg</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -3312,6 +3375,7 @@
       <c r="F19" s="2" t="n">
         <v>6.2878967</v>
       </c>
+      <c r="G19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -3338,6 +3402,7 @@
       <c r="F20" s="2" t="n">
         <v>5.3086679</v>
       </c>
+      <c r="G20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -3364,6 +3429,11 @@
       <c r="F21" s="2" t="n">
         <v>5.5213587</v>
       </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>De Lievekamp</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -3390,6 +3460,11 @@
       <c r="F22" s="2" t="n">
         <v>6.5720279</v>
       </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>SPOT Groningen; SPOT/Stadsschouwburg; Stadsschouwburg Groningen</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -3416,6 +3491,11 @@
       <c r="F23" s="2" t="n">
         <v>4.3627946</v>
       </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Theater de Veste</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -3442,6 +3522,11 @@
       <c r="F24" s="2" t="n">
         <v>5.6174239</v>
       </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Markant; Markant Uden</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -3468,6 +3553,11 @@
       <c r="F25" s="2" t="n">
         <v>4.4586306</v>
       </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Schouwburg De Kring; De Kring Roosendaal</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -3494,6 +3584,11 @@
       <c r="F26" s="2" t="n">
         <v>5.8612019</v>
       </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Toon Hermans Theater Sittard</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -3520,6 +3615,11 @@
       <c r="F27" s="2" t="n">
         <v>5.6614496</v>
       </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Theater Junushoff</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -3546,6 +3646,7 @@
       <c r="F28" s="2" t="n">
         <v>4.7821816</v>
       </c>
+      <c r="G28" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Eerste nieuwe bron via de inleesroutine: Over de liefde van Aaf en Lies, 32 events en 16 nieuwe zalen
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -641,6 +641,46 @@
         <v>3</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Aaf en Lies lossen het wel weer op</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts211/v4/f5/e9/f2/f5e9f2bb-7a5c-f898-cba3-30643cbb762d/mza_1742018322004028896.jpg/600x600bb.png</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Maatschappij</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Aaf Brandt Corstius en Lies Visschedijk maken samen deze podcast van Tonny Media, over de kleine en grote dingen van het dagelijks leven.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Aaf en Lies lossen het wel weer op is de podcast van schrijver Aaf Brandt Corstius en actrice Lies Visschedijk, uitgebracht door Tonny Media. In het theater staan ze met Over de liefde, een voorstelling die in het seizoen 2026 langs ruim twintig Nederlandse theaters reist. LET OP: deze omschrijving is nog summier en moet worden aangevuld.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>1684456730</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -652,7 +692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -754,6 +794,22 @@
           <t>Corti Media Live</t>
         </is>
       </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Over de liefde</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>theatershow</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -766,7 +822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -815,6 +871,14 @@
       </c>
       <c r="B5" s="2" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -828,7 +892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2791,6 +2855,1218 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hnt.nl/nl/voorstellingen/9665/over-de-liefde/aaf-lies</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="n"/>
+      <c r="J46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>https://delamar.nl/voorstellingen/aaf-brandt-corstius-lies-visschedijk/</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="n"/>
+      <c r="J47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>https://delamar.nl/voorstellingen/aaf-brandt-corstius-lies-visschedijk/</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="n"/>
+      <c r="J48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>https://delamar.nl/voorstellingen/aaf-brandt-corstius-lies-visschedijk/</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="n"/>
+      <c r="J49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>https://caprera.nu/programma/aaf-brandt-corstius-en-lies-visschedijk/</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="n"/>
+      <c r="J50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>https://theaterdevest.nl/tickets/seizoen-26-27/aaf-brandt-corstius-lies-visschedijk-over-de-liefde-reprise</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="n"/>
+      <c r="J51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.zwolsetheaters.nl/programma/2025-2026/aaf-brandt-corstius-lies-visschedijk</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="n"/>
+      <c r="J52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>https://leidseschouwburg-stadsgehoorzaal.nl/voorstelling/lies-visschedijk-aaf-brandt-corstius-over-de-liefde-reprise/</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="n"/>
+      <c r="J53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C54" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="n"/>
+      <c r="J54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theateraandeparade.nl/nl/programma/over-de-liefde-aaf-brandt-corstius-lies-visschedijk</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="n"/>
+      <c r="J55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.spotgroningen.nl/programma/aaf-en-lies/</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="n"/>
+      <c r="J56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C57" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dekom.nl/agenda/over-de-liefde-b87t</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="n"/>
+      <c r="J57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kunstmin.nl/voorstellingen/aaf-brandt-corstius-lies-visschedijk-over-de-liefde/</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="n"/>
+      <c r="J58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>https://www.musisenstadstheater.nl/nl/agenda/aaf-brandt-corstius-lies-visschedijk-over-de-liefde/10183</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="n"/>
+      <c r="J59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.schouwburgconcertzaaltilburg.nl/nl/agenda/aaf-lies-over-de-liefde</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="n"/>
+      <c r="J60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.maaspoort.nl/programma/over-de-liefde-aaf-brandt-corstius-lies-visschedijk/17-10-2026-20-15/</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="n"/>
+      <c r="J61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C62" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stadsschouwburgendevereeniging.nl/programma/aaf-brandt-corstius-lies-visschedijk-r342</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="n"/>
+      <c r="J62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C63" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>https://ontdekpoort.nl/programma/2865/aaf-brandt-corstius-lies-visschedijk/</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="n"/>
+      <c r="J63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C64" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>https://www.orpheus.nl/voorstellingen/aaf-brandt-corstius-lies-visschedijk-ns39</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="n"/>
+      <c r="J64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>https://www.chasse.nl/nl/programma/aaf-en-lies-dy3s</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="n"/>
+      <c r="J65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C66" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>https://luxortheater.nl/agenda/aaf-lies-56439</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="n"/>
+      <c r="J66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-11</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>https://hanzehof.nl/nl/voorstelling/aaf-brandt-corstius--lies-visschedijk/</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="n"/>
+      <c r="J67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C68" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.junushoff.nl/programma/aaf-brandt-corstius-lies-visschedijk-l6w1</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="n"/>
+      <c r="J68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-14</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>https://flint.nl/agenda/aaf-brandt-corstius-lies-visschedijk-over-de-liefde/</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="n"/>
+      <c r="J69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-17</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>https://stadstheater.nl/voorstelling/lies-en-aaf/</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="n"/>
+      <c r="J70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C71" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.agnietenhof.nl/agenda/aaf-brandt-corstius-lies-visschedijk-13gr</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="n"/>
+      <c r="J71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C72" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-25</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amphion.nl/theater/aaf-brandt-corstius-lies-visschedijk-over-de-liefde/25-11-2026-20-00/</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="n"/>
+      <c r="J72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-28</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>https://www.spant.org/voorstellingen/over-de-liefde</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="n"/>
+      <c r="J73" s="2" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C74" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>https://kunstlinie.nl/programma/aaf-brandt-corstius-lies-visschedijk/</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="n"/>
+      <c r="J74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-07</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dekleinekomedie.nl/agenda/aaf-brandt-corstius-lies-visschedijk-nrc4</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="n"/>
+      <c r="J75" s="2" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-08</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dekleinekomedie.nl/agenda/aaf-brandt-corstius-lies-visschedijk-nrc4</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="n"/>
+      <c r="J76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-09</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dekleinekomedie.nl/agenda/aaf-brandt-corstius-lies-visschedijk-nrc4</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>https://liesenaaf.nl/</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="n"/>
+      <c r="J77" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2802,7 +4078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3118,7 +4394,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Leidse Schouwburg; Leidse Schouwburg &amp; Stadsgehoorzaal; Stadsgehoorzaal Leiden</t>
+          <t>Stadsgehoorzaal Leiden</t>
         </is>
       </c>
     </row>
@@ -3375,7 +4651,11 @@
       <c r="F19" s="2" t="n">
         <v>6.2878967</v>
       </c>
-      <c r="G19" s="2" t="n"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Schouwburg Amphion</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -3462,7 +4742,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>SPOT Groningen; SPOT/Stadsschouwburg; Stadsschouwburg Groningen</t>
+          <t>SPOT Groningen; SPOT/Stadsschouwburg; Stadsschouwburg Groningen; Stadsschouwburg</t>
         </is>
       </c>
     </row>
@@ -3617,7 +4897,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Theater Junushoff</t>
+          <t>Theater Junushoff; Junushoff</t>
         </is>
       </c>
     </row>
@@ -3646,7 +4926,331 @@
       <c r="F28" s="2" t="n">
         <v>4.7821816</v>
       </c>
-      <c r="G28" s="2" t="n"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Chassé</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Koninklijke Schouwburg</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Den Haag</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Zuid-Holland</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>OLT Caprera</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Bloemendaal</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Holland</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Theater De Vest</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Alkmaar</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Holland</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Leidse Schouwburg</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Leiden</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Zuid-Holland</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>DE KOM</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Nieuwegein</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Utrecht</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Kunstmin</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Dordrecht</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Zuid-Holland</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Maaspoort</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Venlo</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Limburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>De Vereeniging</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Nijmegen</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Gelderland</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Poort</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Sneek</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Friesland</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Orpheus</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Apeldoorn</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Gelderland</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Oude Luxor</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Rotterdam</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Zuid-Holland</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Hanzehof</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Zutphen</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Gelderland</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Flint</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Amersfoort</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Utrecht</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Stadstheater</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Zoetermeer</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Zuid-Holland</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Spant!</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Bussum</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Holland</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>De Kleine Komedie</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Holland</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Alle 43 zalen op de kaart, tijden en prijzen voor wat binnen 90 dagen speelt, drie foute prijzen gecorrigeerd
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -1081,7 +1081,7 @@
         </is>
       </c>
       <c r="I4" s="2" t="n">
-        <v>27</v>
+        <v>12.5</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -1735,7 +1735,7 @@
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
@@ -2803,7 +2803,7 @@
         </is>
       </c>
       <c r="I44" s="2" t="n">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
@@ -2867,7 +2867,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-08 20:00</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2890,7 +2890,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I46" s="2" t="n"/>
+      <c r="I46" s="2" t="n">
+        <v>14.5</v>
+      </c>
       <c r="J46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
@@ -2905,7 +2907,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-11 20:30</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2915,7 +2917,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>in verkoop</t>
+          <t>uitverkocht</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -2928,7 +2930,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I47" s="2" t="n"/>
+      <c r="I47" s="2" t="n">
+        <v>19.5</v>
+      </c>
       <c r="J47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
@@ -2943,7 +2947,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-12 20:30</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2953,7 +2957,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>in verkoop</t>
+          <t>uitverkocht</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -2966,7 +2970,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I48" s="2" t="n"/>
+      <c r="I48" s="2" t="n">
+        <v>19.5</v>
+      </c>
       <c r="J48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
@@ -2981,7 +2987,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-13 14:30</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -3004,7 +3010,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I49" s="2" t="n"/>
+      <c r="I49" s="2" t="n">
+        <v>19.5</v>
+      </c>
       <c r="J49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
@@ -3019,7 +3027,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-17 20:30</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -3042,7 +3050,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I50" s="2" t="n"/>
+      <c r="I50" s="2" t="n">
+        <v>32.5</v>
+      </c>
       <c r="J50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
@@ -3133,7 +3143,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-23 20:15</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -3156,7 +3166,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I53" s="2" t="n"/>
+      <c r="I53" s="2" t="n">
+        <v>29.5</v>
+      </c>
       <c r="J53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
@@ -3205,7 +3217,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-27 20:30</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -3228,7 +3240,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I55" s="2" t="n"/>
+      <c r="I55" s="2" t="n">
+        <v>13.5</v>
+      </c>
       <c r="J55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
@@ -3243,7 +3257,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-04 20:15</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -3281,7 +3295,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-07 20:15</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -3304,7 +3318,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I57" s="2" t="n"/>
+      <c r="I57" s="2" t="n">
+        <v>29</v>
+      </c>
       <c r="J57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
@@ -3319,7 +3335,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-08 20:00</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -3342,7 +3358,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I58" s="2" t="n"/>
+      <c r="I58" s="2" t="n">
+        <v>27</v>
+      </c>
       <c r="J58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
@@ -3357,7 +3375,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-15 20:00</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -3380,7 +3398,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I59" s="2" t="n"/>
+      <c r="I59" s="2" t="n">
+        <v>18</v>
+      </c>
       <c r="J59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
@@ -3395,7 +3415,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-16 20:15</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -3418,7 +3438,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I60" s="2" t="n"/>
+      <c r="I60" s="2" t="n">
+        <v>24.5</v>
+      </c>
       <c r="J60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
@@ -3433,7 +3455,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-17 20:15</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -3456,7 +3478,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I61" s="2" t="n"/>
+      <c r="I61" s="2" t="n">
+        <v>26</v>
+      </c>
       <c r="J61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
@@ -3471,7 +3495,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-20 20:15</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3494,7 +3518,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I62" s="2" t="n"/>
+      <c r="I62" s="2" t="n">
+        <v>31</v>
+      </c>
       <c r="J62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
@@ -3509,7 +3535,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-22 20:15</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -3532,7 +3558,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I63" s="2" t="n"/>
+      <c r="I63" s="2" t="n">
+        <v>29.5</v>
+      </c>
       <c r="J63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
@@ -3547,7 +3575,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-27 20:00</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3570,7 +3598,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I64" s="2" t="n"/>
+      <c r="I64" s="2" t="n">
+        <v>26</v>
+      </c>
       <c r="J64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
@@ -3585,7 +3615,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-30 20:00</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -3595,7 +3625,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>in verkoop</t>
+          <t>uitverkocht</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -3608,7 +3638,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I65" s="2" t="n"/>
+      <c r="I65" s="2" t="n">
+        <v>18</v>
+      </c>
       <c r="J65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
@@ -3623,7 +3655,7 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>2026-11-04</t>
+          <t>2026-11-04 20:00</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -3646,7 +3678,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I66" s="2" t="n"/>
+      <c r="I66" s="2" t="n">
+        <v>18.5</v>
+      </c>
       <c r="J66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
@@ -3699,7 +3733,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-11-12 20:15</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -3722,7 +3756,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I68" s="2" t="n"/>
+      <c r="I68" s="2" t="n">
+        <v>30.5</v>
+      </c>
       <c r="J68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
@@ -3737,7 +3773,7 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>2026-11-14</t>
+          <t>2026-11-14 20:15</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -3760,7 +3796,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I69" s="2" t="n"/>
+      <c r="I69" s="2" t="n">
+        <v>24</v>
+      </c>
       <c r="J69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
@@ -3775,7 +3813,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>2026-11-17</t>
+          <t>2026-11-17 20:00</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -3798,7 +3836,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I70" s="2" t="n"/>
+      <c r="I70" s="2" t="n">
+        <v>32</v>
+      </c>
       <c r="J70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
@@ -3813,7 +3853,7 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-11-19 20:00</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -3836,7 +3876,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I71" s="2" t="n"/>
+      <c r="I71" s="2" t="n">
+        <v>31</v>
+      </c>
       <c r="J71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
@@ -3851,7 +3893,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>2026-11-25</t>
+          <t>2026-11-25 20:00</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -3874,7 +3916,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I72" s="2" t="n"/>
+      <c r="I72" s="2" t="n">
+        <v>30</v>
+      </c>
       <c r="J72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
@@ -3889,7 +3933,7 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-11-28 20:15</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -3912,7 +3956,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I73" s="2" t="n"/>
+      <c r="I73" s="2" t="n">
+        <v>31.5</v>
+      </c>
       <c r="J73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
@@ -4951,6 +4997,13 @@
           <t>Zuid-Holland</t>
         </is>
       </c>
+      <c r="E29" s="2" t="n">
+        <v>52.0818859</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>4.3158207</v>
+      </c>
+      <c r="G29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -4971,6 +5024,17 @@
           <t>Noord-Holland</t>
         </is>
       </c>
+      <c r="E30" s="2" t="n">
+        <v>52.4112527</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>4.6060681</v>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Openluchttheater Caprera; Caprera</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -4991,6 +5055,17 @@
           <t>Noord-Holland</t>
         </is>
       </c>
+      <c r="E31" s="2" t="n">
+        <v>52.6338681</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>4.7439242</v>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>De Vest</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -5011,6 +5086,13 @@
           <t>Zuid-Holland</t>
         </is>
       </c>
+      <c r="E32" s="2" t="n">
+        <v>52.1621894</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>4.4891831</v>
+      </c>
+      <c r="G32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -5031,6 +5113,17 @@
           <t>Utrecht</t>
         </is>
       </c>
+      <c r="E33" s="2" t="n">
+        <v>52.0273057</v>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>5.0849865</v>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>De Kom; Theater De Kom</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -5051,6 +5144,17 @@
           <t>Zuid-Holland</t>
         </is>
       </c>
+      <c r="E34" s="2" t="n">
+        <v>51.8139254</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>4.6764483</v>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Schouwburg Kunstmin</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -5071,6 +5175,17 @@
           <t>Limburg</t>
         </is>
       </c>
+      <c r="E35" s="2" t="n">
+        <v>51.3703643</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>6.1678835</v>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>De Maaspoort; Theater de Maaspoort</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -5091,6 +5206,17 @@
           <t>Gelderland</t>
         </is>
       </c>
+      <c r="E36" s="2" t="n">
+        <v>51.8412654</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>5.8611299</v>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Concertgebouw de Vereeniging; De Vereeniging</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -5111,6 +5237,17 @@
           <t>Friesland</t>
         </is>
       </c>
+      <c r="E37" s="2" t="n">
+        <v>53.0317815</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>5.6562252</v>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Theater Sneek</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -5131,6 +5268,17 @@
           <t>Gelderland</t>
         </is>
       </c>
+      <c r="E38" s="2" t="n">
+        <v>52.2197051</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>5.9529526</v>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Theater Orpheus</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -5151,6 +5299,17 @@
           <t>Zuid-Holland</t>
         </is>
       </c>
+      <c r="E39" s="2" t="n">
+        <v>51.9229973</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>4.4770274</v>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Oude Luxor theater; Oude Luxor Theater</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -5171,6 +5330,17 @@
           <t>Gelderland</t>
         </is>
       </c>
+      <c r="E40" s="2" t="n">
+        <v>52.148269</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>6.2017651</v>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Theater Hanzehof</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -5191,6 +5361,17 @@
           <t>Utrecht</t>
         </is>
       </c>
+      <c r="E41" s="2" t="n">
+        <v>52.1595514</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>5.3928003</v>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>De Flint; Theater Flint</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -5211,6 +5392,17 @@
           <t>Zuid-Holland</t>
         </is>
       </c>
+      <c r="E42" s="2" t="n">
+        <v>52.0623265</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>4.4937402</v>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Stadstheater Zoetermeer</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -5231,6 +5423,17 @@
           <t>Noord-Holland</t>
         </is>
       </c>
+      <c r="E43" s="2" t="n">
+        <v>52.2700169</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>5.1751674</v>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Spant</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -5251,6 +5454,13 @@
           <t>Noord-Holland</t>
         </is>
       </c>
+      <c r="E44" s="2" t="n">
+        <v>52.3669037</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>4.8960251</v>
+      </c>
+      <c r="G44" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Toplijst houdt nu bij wat is nagekeken: drie toestanden en een voortgangsteller
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="show_podcasts" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="events" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="venues" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="toplijst" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5465,4 +5466,2480 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G101"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>apple_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>rang</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>naam</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>maker</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>gecontroleerd_op</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>bevinding</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>notitie</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1513807137</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Maarten van Rossem &amp; Tom Jessen</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Tom Jessen en Maarten van Rossem</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>De Verkiezingsshow speelde 7 okt 2025 in Den Haag, geweest; niets nieuws in verkoop</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>6802611523</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Schuilen in Schoonheid</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Dag &amp; Nacht</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>1076289388</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Boekestijn en De Wijk</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>BNR Nieuwsradio</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Corti Media, eindejaarsshow 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>6802583563</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>De Wit &amp; De Wereld</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / BNNVARA</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>1202584124</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>De Stemming van Vullings en De Rooy</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>NPO Radio 1 / NOS / EenVandaag</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>geen theatervoorstelling gevonden</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>6805798686</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Belleman &amp; Van Dop</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / BNNVARA</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>nieuwe misdaadpodcast, geen voorstelling gevonden</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>1684456730</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Aaf en Lies lossen het wel weer op</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Tonny Media</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>1334620583</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>De Jortcast</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / AVROTROS</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>1551138207</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>de Volkskrant Elke Dag</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>de Volkskrant</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>1460234936</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>NRC Vandaag</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>NRC</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>1591011702</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Napleiten</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Wouter Laumans, Christian Flokstra</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Corti Media, tour t/m mei 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>1458702219</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>De Ongelooflijke Podcast</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / EO</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>204558483</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>NOS Met het Oog op Morgen</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>NPO Radio 1 / NOS</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>1478135753</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Amerika in 15 minuten</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Raymond Mens</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>1606935703</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Vandaag Inside</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Vandaag Inside</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>1339219119</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>De Dag</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / NOS</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>1520628483</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Parool Misdaadpodcast</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Het Parool</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>1824643677</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Verdwenen</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / EO</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>1546378955</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Marc-Marie &amp; Isa Vinden Iets</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Marc-Marie &amp; Isa / Tonny Media</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>een zoekopdracht, geen theatertour gevonden</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>1609407191</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Reality Check - B&amp;B Vol Liefde</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Dag en Nacht</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>1753702871</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Moorden in de jaren...</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Hanneke Hendrix &amp; Lotte Lentes / New Tree Media</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>1458606160</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>De Publieke Tribune</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>NPO Radio 1 / HUMAN</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>1858969277</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Heterdaad</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>De Telegraaf</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>1643003287</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>NRC Het Uur</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>NRC</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>1449765297</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>De Nieuwe Wereld</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>De Nieuwe Wereld</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>793155061</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Nooit meer slapen</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>NPO Radio 1 / VPRO</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>1537788786</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>The Rest Is History</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Goalhanger</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>1869672584</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Provinfluencers</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Plien &amp; Bianca/Tonny Media</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>TWIJFEL: Plien &amp; Bianca spelen Harrekidee!, maar dat is cabaret en gaat niet over de podcast</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>1596318678</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>De Grote Podcastlas</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Leon Boelens, Max Gerritsen &amp; Hugo Noordman</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>1599086196</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>FD Dagkoers</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Het Financieele Dagblad</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>1454364435</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Kick-off met Valentijn Driessen</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>De Telegraaf</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>1493941133</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Blokhuis de Podcast</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / BNNVARA</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>1607083067</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Weer een dag</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Marcel van Roosmalen &amp; Gijs Groenteman / Meer van dit</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>geen actuele tour gevonden; laatste theateroptreden dateert van eerder</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>1503500354</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>RADIO BOOS</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / BNNVARA</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>1310805889</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Met Groenteman in de kast</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>de Volkskrant</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>1621278264</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Alle Geschiedenis Ooit - Grote Namen</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Alle Geschiedenis Ooit</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>1731378143</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>KieftJansenEgmondGijp</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>KieftJansenEgmondGijp</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>1511727831</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Afhameren met Wouter de Winther</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>De Telegraaf</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>1423659847</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Omdenken Podcast</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Berthold Gunster</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>LEAD: Berthold Gunster heeft een lopende theatershow via omdenken.nl - nog uitzoeken</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>1509692709</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Geschiedenis voor herbeginners</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Jonas Goossenaerts e.a.</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr"/>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>1586453689</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Victor Duidt TV</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Victor Vlam</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>1205520865</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>NRC Haagse Zaken</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>NRC</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>1397767808</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>AD Voetbal podcast</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>AD</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>1425829411</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>NOS Voetbalpodcast</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / NOS</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr"/>
+      <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>1385505692</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>De Universiteit van Nederland Podcast</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Universiteit van Nederland</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>LEAD: Universiteit van Nederland LIVE - Wetenschap voor iedereen, tourt - nog uitzoeken</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>1692318247</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>AI Report</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Alexander Klopping en Wietse Hage</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>1709945407</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>NOS Wielerpodcast</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / NOS</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>1434702387</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Betrouwbare Bronnen</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Jaap Jansen - Dag en Nacht Media</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>1465937226</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Amerika Podcast</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>BNR Nieuwsradio</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>1541475237</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Teun en Gijs vertellen alles</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Teun van de Keuken &amp; Gijs Groenteman / Meer van dit</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>1665930221</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>De Zaak X</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>AD</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>1361193085</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>In Het Wiel</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>DPG Media</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr"/>
+      <c r="F53" s="2" t="inlineStr"/>
+      <c r="G53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>1790654002</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Scientias Podcast</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Scientias</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>1706997830</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>B&amp;B Vol Liefde 2026: De Nabeschouwing</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Veronica Superguide</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr"/>
+      <c r="F55" s="2" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>6799945485</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>We call her Emma</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>The Observer</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>1854108027</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>De Ware Jacob</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Dagblad van het Noorden</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>1896787047</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Ontvoerd naar Noord-Korea</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>De Telegraaf</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>638203140</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Echt Gebeurd</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Echt Gebeurd</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr"/>
+      <c r="G59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>1615734652</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>De Saarpodcast</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Saar Magazine</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>1889109038</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Even Denken</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Universiteit van Nederland / Podimo</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>1867183750</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Tina FM: B&amp;B Vol Liefde</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Audiohuis</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>1412808006</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>VPRO Zomergasten</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / VPRO</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr"/>
+      <c r="G63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>1890465212</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>De Onderwereld</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Bas Dingemanse &amp; Bas van Mulken</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr"/>
+      <c r="G64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>1637601065</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>VI ZSM</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Voetbal International</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr"/>
+      <c r="F65" s="2" t="inlineStr"/>
+      <c r="G65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>1529310093</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Pak Schaal Podcast</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Voetbal International</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr"/>
+      <c r="G66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>1444731970</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Zembla Podcast: Op zoek naar Marlotte</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / BNNVARA</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr"/>
+      <c r="F67" s="2" t="inlineStr"/>
+      <c r="G67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>6786336779</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Zwijgen aan Zee</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / BNNVARA</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr"/>
+      <c r="G68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>1755711498</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Trias Criminalis</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Marian Husken, John Pel &amp; Mark Teurlings / Audiohuis</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr"/>
+      <c r="F69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>1334611654</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Nieuwsweekend</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>NPO Radio 1 / Omroep MAX</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr"/>
+      <c r="G70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>1481398762</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Dolly Parton's America</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>WNYC Studios &amp; OSM Audio</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr"/>
+      <c r="F71" s="2" t="inlineStr"/>
+      <c r="G71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>1501959067</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Wat een Week!</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Maxim Hartman &amp; Willem Treur</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr"/>
+      <c r="G72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>1746899086</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Geschiedenis Inside</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Tonny Media</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr"/>
+      <c r="F73" s="2" t="inlineStr"/>
+      <c r="G73" s="2" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>1200361736</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>The Daily</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>The New York Times</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr"/>
+      <c r="G74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>1534035895</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Ervaring voor Beginners</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Comedytrain</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="inlineStr"/>
+      <c r="G75" s="2" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>1745655944</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Hedy &amp; Hadassah - Vrolijk Voorwaarts</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Hadassah de Boer</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr"/>
+      <c r="G76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>1529796628</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Moordzaken</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Carrie &amp; Eddie</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr"/>
+      <c r="F77" s="2" t="inlineStr"/>
+      <c r="G77" s="2" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>1447850163</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>F1 Aan Tafel</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Grand Prix Radio</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>1807335832</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Daphne's Hulptroepen</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Dag en Nacht / Podimo</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="inlineStr"/>
+      <c r="G79" s="2" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>1361734727</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>NRC Onbehaarde Apen</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>NRC</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr"/>
+      <c r="F80" s="2" t="inlineStr"/>
+      <c r="G80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>1807039003</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Verraad in de geschiedenis</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>David Lucieer, Thom Aalmoes &amp; Elisabeth Hoekstra / New Tree Media</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr"/>
+      <c r="G81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>1399043180</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Voetbalpraat</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>ESPN NL</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr"/>
+      <c r="G82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>1890178832</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>De Vondeling</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>AT5</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr"/>
+      <c r="F83" s="2" t="inlineStr"/>
+      <c r="G83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>1842312260</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Het Spreekuur</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Erik Scherder, Leonard Hofstra, Brechje van Bladel / Corti Media &amp; Quest</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr"/>
+      <c r="G84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>1823118868</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Radio Romano</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Marcel van Roosmalen, Noortje Veldhuizen &amp; Roelof de Vries</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr"/>
+      <c r="F85" s="2" t="inlineStr"/>
+      <c r="G85" s="2" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>985794392</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Bureau Buitenland</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>NPO Radio 1 / VPRO</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr"/>
+      <c r="G86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>1673350701</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Veldheren</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>Peter van Uhm, Mart de Kruif, Jos de Groot / Corti Media</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="inlineStr"/>
+      <c r="G87" s="2" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>1895913555</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Bokkenrijders</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Toneelgroep Maastricht en L1</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr"/>
+      <c r="G88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>1548342984</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Geuze &amp; Gorgels</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>Monica &amp; Kaj / Tonny Media</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>een zoekopdracht, geen theatertour gevonden</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>6792748139</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Patrick en Eline</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Patrick en Eline</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="inlineStr"/>
+      <c r="G90" s="2" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>1740313422</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Chantal &amp; Tina</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>&amp;C Media / Audiohuis</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr"/>
+      <c r="F91" s="2" t="inlineStr"/>
+      <c r="G91" s="2" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>1166206395</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>De Wereld - BNR</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>BNR Nieuwsradio</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr"/>
+      <c r="G92" s="2" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>1447387615</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>De Brand in het Landhuis</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / NTR</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr"/>
+      <c r="G93" s="2" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>1438232918</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Het Land van Wierd Duk</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>De Telegraaf</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="inlineStr"/>
+      <c r="G94" s="2" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>1635098263</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>In de ban van Rian</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>AD / Tubantia</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr"/>
+      <c r="G95" s="2" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>1553924343</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Het Misdaadbureau</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / PowNed</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr"/>
+      <c r="G96" s="2" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>1602986598</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>MISCHA!</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / AVROTROS</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="inlineStr"/>
+      <c r="G97" s="2" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>1845304226</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Rechtpraten</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Royce de Vries &amp; Annemiek van Spanje / New Tree Media</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr"/>
+      <c r="G98" s="2" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>924429487</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>De Correspondent</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>De Correspondent</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr"/>
+      <c r="F99" s="2" t="inlineStr"/>
+      <c r="G99" s="2" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>1684893613</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Van Bekhovens Britten - BNR</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>BNR Nieuwsradio</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr"/>
+      <c r="F100" s="2" t="inlineStr"/>
+      <c r="G100" s="2" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>1479010914</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Europa Draait Door</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>NPO Luister / VPRO</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr"/>
+      <c r="F101" s="2" t="inlineStr"/>
+      <c r="G101" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Afbakeningsregel vastgelegd met kolom verwantschap; Harrekidee van Plien en Bianca toegevoegd, 42 events en 17 zalen
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -682,6 +682,46 @@
         <v>7</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Provinfluencers</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts211/v4/91/3d/c2/913dc24a-2ebd-751e-ebd4-72387685e003/mza_5988287602256490768.jpg/600x600bb.png</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Comedy</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Plien van Bennekom en Bianca Krijgsman maken samen Provinfluencers, een komische podcast van Tonny Media.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Provinfluencers is de podcast van Plien van Bennekom en Bianca Krijgsman, uitgebracht door Tonny Media en te vinden in de Nederlandse podcast top 100. In het theater staan ze met de reprise van Harrekidee!, hun cabaretvoorstelling, die in het seizoen 2026-2027 langs ruim dertig theaters reist. Die voorstelling komt niet uit de podcast voort, maar wordt door hetzelfde duo gespeeld in dezelfde toon. LET OP: deze omschrijving is nog summier en moet worden aangevuld.</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>1869672584</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -693,13 +733,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -723,6 +764,11 @@
           <t>organisator</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>verwantschap</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -739,6 +785,11 @@
         </is>
       </c>
       <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>podcast live</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -759,6 +810,11 @@
           <t>Corti Media Live i.s.m. BNR</t>
         </is>
       </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>thema-verwant</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -775,6 +831,11 @@
         </is>
       </c>
       <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>thema-verwant</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -795,6 +856,11 @@
           <t>Corti Media Live</t>
         </is>
       </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>thema-verwant</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -811,6 +877,36 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>zelfde makers</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Harrekidee! (reprise)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>theatershow</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Bos Theaterproducties</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>zelfde makers</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -823,7 +919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -880,6 +976,14 @@
       </c>
       <c r="B6" s="2" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -893,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4114,6 +4218,1506 @@
       <c r="I77" s="2" t="n"/>
       <c r="J77" s="2" t="inlineStr"/>
     </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="n"/>
+      <c r="J78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="n"/>
+      <c r="J79" s="2" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C80" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theateraandeparade.nl/nl/programma/plien-en-bianca-harrekidee-reprise</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="n"/>
+      <c r="J80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>https://theaterdevest.nl/tickets/seizoen-26-27/plien-bianca-harrekidee-reprise</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="n"/>
+      <c r="J81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="n"/>
+      <c r="J82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C83" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr"/>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="n"/>
+      <c r="J83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C84" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="n"/>
+      <c r="J84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C85" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr"/>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="n"/>
+      <c r="J85" s="2" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C86" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="n"/>
+      <c r="J86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C87" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="n"/>
+      <c r="J87" s="2" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C88" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="n"/>
+      <c r="J88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C89" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hnt.nl/nl/voorstellingen/plien-bianca-7w3w</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="n"/>
+      <c r="J89" s="2" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C90" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="n"/>
+      <c r="J90" s="2" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C91" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr"/>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="n"/>
+      <c r="J91" s="2" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C92" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="n"/>
+      <c r="J92" s="2" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C93" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="n"/>
+      <c r="J93" s="2" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C94" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>https://www.spant.org/voorstellingen/plien-bianca</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="n"/>
+      <c r="J94" s="2" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C95" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theaterroermond.nl/agenda/plien-bianca-reprise</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="n"/>
+      <c r="J95" s="2" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C96" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="n"/>
+      <c r="J96" s="2" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C97" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="n"/>
+      <c r="J97" s="2" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C98" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="n"/>
+      <c r="J98" s="2" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C99" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr"/>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="n"/>
+      <c r="J99" s="2" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C100" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>https://www.spotgroningen.nl/programma/plien-bianca-8/</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="n"/>
+      <c r="J100" s="2" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C101" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr"/>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="n"/>
+      <c r="J101" s="2" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C102" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-05</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr"/>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="n"/>
+      <c r="J102" s="2" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C103" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>https://www.atlastheater.nl/voorstellingen/harrekidee-reprise-plien-en-bianca-09-nov/</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="n"/>
+      <c r="J103" s="2" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C104" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>https://www.wilminktheater.nl/nl/agenda/harrekidee-herneming-yw51</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="n"/>
+      <c r="J104" s="2" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C105" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr"/>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="n"/>
+      <c r="J105" s="2" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C106" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr"/>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="n"/>
+      <c r="J106" s="2" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C107" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-17</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr"/>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="n"/>
+      <c r="J107" s="2" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C108" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>https://www.maaspoort.nl/programma/harrekidee-reprise-plien-bianca/19-11-2026-20-15/</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="n"/>
+      <c r="J108" s="2" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C109" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-23</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>https://www.chasse.nl/nl/programma/plien-bianca-l914</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="n"/>
+      <c r="J109" s="2" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C110" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-24</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>https://www.zeelandtheaters.nl/programma/plien-bianca-harrekidee-reprise/24-11-2026-20-00</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="n"/>
+      <c r="J110" s="2" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C111" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-26</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>https://www.demaagd.nl/agenda/plien-en-bianca-t2gz</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="n"/>
+      <c r="J111" s="2" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C112" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr"/>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="n"/>
+      <c r="J112" s="2" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C113" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theaterdeveste.nl/programma/harrekidee-68ky</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="n"/>
+      <c r="J113" s="2" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C114" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-03</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr"/>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="n"/>
+      <c r="J114" s="2" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C115" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-07</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>https://www.afastheater.nl/plien-en-bianca</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I115" s="2" t="n"/>
+      <c r="J115" s="2" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C116" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-08</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>https://www.afastheater.nl/plien-en-bianca</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="n"/>
+      <c r="J116" s="2" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C117" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-09</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>https://www.afastheater.nl/plien-en-bianca</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="n"/>
+      <c r="J117" s="2" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C118" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-15</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>https://luxortheater.nl/agenda/plien-bianca-57558</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="n"/>
+      <c r="J118" s="2" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C119" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>https://luxortheater.nl/agenda/plien-bianca-57558</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>https://plienenbianca.nl/speellijsten/</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I119" s="2" t="n"/>
+      <c r="J119" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4125,7 +5729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5462,6 +7066,509 @@
         <v>4.8960251</v>
       </c>
       <c r="G44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Theater Lampegiet</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Veenendaal</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Utrecht</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>52.0244718</v>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>5.5529666</v>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Theater De Lampegiet; De Lampegiet</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Deventer Schouwburg</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Deventer</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Overijssel</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>52.2556465</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>6.1615569</v>
+      </c>
+      <c r="G46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Schouwburg Cuijk</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Cuijk</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Brabant</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>51.7282504</v>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>5.8819203</v>
+      </c>
+      <c r="G47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>De Rijswijkse Schouwburg</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Rijswijk</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Zuid-Holland</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>52.0460579</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>4.327609</v>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Rijswijkse Schouwburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Theater De Oranjerie</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Roermond</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Limburg</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>51.1916778</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>5.9896043</v>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Theaterhotel De Oranjerie; De Oranjerie</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Cool Kunst en Cultuur</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Heerhugowaard</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Holland</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>52.6623256</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>4.82789</v>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Cool</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Theater De Tamboer</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Hoogeveen</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Drenthe</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>52.7273643</v>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>6.4779898</v>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>De Tamboer</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Zaantheater</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Zaandam</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Holland</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>52.4382663</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>4.824913</v>
+      </c>
+      <c r="G52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Theater DNK</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Assen</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Drenthe</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>52.9947861</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>6.5582666</v>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>De Nieuwe Kolk; DNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>ATLAS Theater</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Emmen</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Drenthe</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>52.7830595</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>6.891167</v>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Atlas Theater</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Wilminktheater</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Enschede</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Overijssel</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>52.2226746</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>6.8947417</v>
+      </c>
+      <c r="G55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>De Blauwe Kei</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Veghel</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Brabant</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>51.6148637</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>5.5298913</v>
+      </c>
+      <c r="G56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Schouwburg De Lawei</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Drachten</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Friesland</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>53.1031073</v>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>6.0985494</v>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>De Lawei</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Scheldetheater</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Terneuzen</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Zeeland</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>51.3386553</v>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>3.8231688</v>
+      </c>
+      <c r="G58" s="2" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Theater De Maagd</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Bergen op Zoom</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Brabant</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>51.4942791</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>4.2861736</v>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>De Maagd</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Agora Theater</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Lelystad</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Flevoland</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>52.5108687</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>5.4763167</v>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Agora Theater en Congrescentrum; Agora</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>AFAS Theater Leusden</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Leusden</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Utrecht</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>52.1419261</v>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>5.4211143</v>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>AFAS Theater</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6243,11 +8350,19 @@
           <t>Plien &amp; Bianca/Tonny Media</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr"/>
-      <c r="F29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>liveshow gevonden</t>
+        </is>
+      </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>TWIJFEL: Plien &amp; Bianca spelen Harrekidee!, maar dat is cabaret en gaat niet over de podcast</t>
+          <t>Harrekidee! (reprise) via plienenbianca.nl - verwantschap: zelfde makers</t>
         </is>
       </c>
     </row>
@@ -6512,11 +8627,19 @@
           <t>Berthold Gunster</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>LEAD: Berthold Gunster heeft een lopende theatershow via omdenken.nl - nog uitzoeken</t>
+          <t>theatershow Zoals verwacht loopt alles anders is in 2026 afgelopen, geen nieuwe data</t>
         </is>
       </c>
     </row>
@@ -6658,7 +8781,7 @@
       <c r="F46" s="2" t="inlineStr"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>LEAD: Universiteit van Nederland LIVE - Wetenschap voor iedereen, tourt - nog uitzoeken</t>
+          <t>LEAD: Universiteit van Nederland LIVE tourt, speellijst nog niet gevonden</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Parool Misdaadpodcast toegevoegd: De Misdaadpodcast Live, 6 data uit losse theaterpaginas
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -722,6 +722,46 @@
         <v>28</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Parool Misdaadpodcast</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts211/v4/c8/21/b3/c821b3a4-aa7c-2418-0f56-472f093efacd/mza_10406733572000608125.jpg/600x600bb.png</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>True crime</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Misdaadverslaggevers van Het Parool bespreken de Amsterdamse onderwereld en de strafzaken die daaruit voortkomen.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>De Parool Misdaadpodcast wordt gemaakt door misdaadjournalisten van Het Parool en staat in de Nederlandse podcast top 100. In het theater spelen Paul Vugts, Wouter Laumans en Corrie Gerritsma De Misdaadpodcast Live, waarin ze zaken uit hun vakgebied voor publiek uitdiepen. Wouter Laumans staat ook in Napleiten Live. LET OP: deze omschrijving is nog summier en moet worden aangevuld.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>1520628483</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -733,7 +773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -908,6 +948,27 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>De Misdaadpodcast Live</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>theatershow</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>thema-verwant</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -919,7 +980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -984,6 +1045,14 @@
       </c>
       <c r="B7" s="2" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -997,7 +1066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J119"/>
+  <dimension ref="A1:J125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5718,6 +5787,234 @@
       <c r="I119" s="2" t="n"/>
       <c r="J119" s="2" t="inlineStr"/>
     </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C120" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 20:00</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theateraandeparade.nl/nl/programma/misdaadpodcast-live</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theateraandeparade.nl/nl/programma/misdaadpodcast-live</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="J120" s="2" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C121" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-20 20:00</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>https://luxortheater.nl/agenda/de-misdaadpodcast-live-58250</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>https://luxortheater.nl/agenda/de-misdaadpodcast-live-58250</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I121" s="2" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="J121" s="2" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C122" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-10 20:15</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr"/>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theater.nl/de-misdaadpodcast-live-paul-vugts-wouter-laumans-en-corrie-gerritsma</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="n"/>
+      <c r="J122" s="2" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C123" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-05 20:00</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>https://www.orpheus.nl/voorstellingen/de-misdaadpodcast-live-97vl</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>https://www.orpheus.nl/voorstellingen/de-misdaadpodcast-live-97vl</t>
+        </is>
+      </c>
+      <c r="H123" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I123" s="2" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="J123" s="2" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C124" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>2027-04-13 20:00</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theateraanhetvrijthof.nl/voorstellingen/theatercollege-en-literair/met-paul-vugts-wouter-laumans-en-corrie-gerritsma-de-misdaadpodcast-live</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theateraanhetvrijthof.nl/voorstellingen/theatercollege-en-literair/met-paul-vugts-wouter-laumans-en-corrie-gerritsma-de-misdaadpodcast-live</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I124" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="J124" s="2" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C125" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>2027-05-27 20:15</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr"/>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theater.nl/de-misdaadpodcast-live-paul-vugts-wouter-laumans-en-corrie-gerritsma</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I125" s="2" t="n"/>
+      <c r="J125" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5729,7 +6026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7567,6 +7864,99 @@
       <c r="G61" s="2" t="inlineStr">
         <is>
           <t>AFAS Theater</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Cultuurhuis De Klinker</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Winschoten</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Groningen</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>53.1472327</v>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>7.033705</v>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>De Klinker</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Theater aan het Vrijthof</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Maastricht</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Limburg</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="n">
+        <v>50.8502223</v>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>5.6879791</v>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Vrijthof</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Schouwburg Het Park</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Hoorn</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Holland</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>52.6416444</v>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>5.0512565</v>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Het Park</t>
         </is>
       </c>
     </row>
@@ -8085,9 +8475,21 @@
           <t>Het Parool</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>De Misdaadpodcast Live, 6 data gevonden via losse theaterpagina's; geen centrale speellijst, lijst mogelijk incompleet</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Corti Media live-shows toegevoegd + Parool-misdaadpodcast aangevuld
- Best of 'Help, ik heb een Puber' (5 data) en ontbrekende data bij
  Boekestijn & De Wijk Live toegevoegd via cortimedia.nl/live
- Parool webwinkel gebruikt om prijzen Winschoten/Hoorn aan te vullen
  en de misdaadpodcast-tour te bevestigen als 8 data (2 nog zonder
  bekende zaalnaam)
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -762,6 +762,41 @@
         <v>17</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Help, ik word volwassen!</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts221/v4/a0/1b/c4/a01bc439-71a8-107c-9d17-d667df42192b/mza_4432722255828391472.jpg/600x600bb.jpg</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.cortimedia.nl/help-ik-heb-een-puber</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Opvoeding</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Kluun en Yvanka van der Zwaan bespreken wekelijks de uitdagingen van het opvoeden van pubers - herkenbaar, eerlijk en met humor. De podcast heette eerder 'Help, ik heb een puber!'.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>1726575117</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -773,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -969,6 +1004,31 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Best of 'Help, ik heb een Puber'</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>theatershow</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Corti Media</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>podcast live</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -980,7 +1040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1053,6 +1113,14 @@
       </c>
       <c r="B8" s="2" t="n">
         <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1066,7 +1134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J125"/>
+  <dimension ref="A1:J132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2377,7 +2445,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="I30" s="2" t="n"/>
@@ -2419,7 +2487,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="I31" s="2" t="n">
@@ -2507,7 +2575,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="I33" s="2" t="n">
@@ -2547,7 +2615,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2651,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="I35" s="2" t="n"/>
@@ -2621,7 +2689,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="I36" s="2" t="n">
@@ -2665,7 +2733,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="I37" s="2" t="n">
@@ -2753,7 +2821,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="I39" s="2" t="n">
@@ -2797,7 +2865,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="I40" s="2" t="n">
@@ -2841,7 +2909,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="I41" s="2" t="n">
@@ -2885,7 +2953,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="I42" s="2" t="n">
@@ -2929,7 +2997,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="I43" s="2" t="n">
@@ -2973,7 +3041,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="I44" s="2" t="n">
@@ -3017,7 +3085,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="I45" s="2" t="n">
@@ -5898,7 +5966,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I122" s="2" t="n"/>
+      <c r="I122" s="2" t="n">
+        <v>25.5</v>
+      </c>
       <c r="J122" s="2" t="inlineStr"/>
     </row>
     <row r="123">
@@ -6012,8 +6082,276 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I125" s="2" t="n"/>
+      <c r="I125" s="2" t="n">
+        <v>29.5</v>
+      </c>
       <c r="J125" s="2" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C126" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 20:15</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lievekamp.nl/programma/met-kluun-yvanka-van-der-zwaan-the-best-of-help-ik-heb-een-puber-07-okt-20-15/</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lievekamp.nl/programma/met-kluun-yvanka-van-der-zwaan-the-best-of-help-ik-heb-een-puber-07-okt-20-15/</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J126" s="2" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C127" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28 20:30</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>https://delamar.nl/voorstellingen/best-of-help-ik-heb-een-puber-live/</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>https://delamar.nl/voorstellingen/best-of-help-ik-heb-een-puber-live/</t>
+        </is>
+      </c>
+      <c r="H127" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I127" s="2" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="J127" s="2" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C128" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 20:15</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>https://www.spotgroningen.nl/programma/kluun-en-yvanka-van-der-zwaan/</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>https://www.spotgroningen.nl/programma/kluun-en-yvanka-van-der-zwaan/</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J128" s="2" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C129" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-25 20:00</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>https://www.schouwburgconcertzaaltilburg.nl/nl/agenda/kluun-help-ik-heb-een-puber</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>https://www.schouwburgconcertzaaltilburg.nl/nl/agenda/kluun-help-ik-heb-een-puber</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I129" s="2" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J129" s="2" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C130" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theateraandeparade.nl/nl/programma/the-best-of-help-ik-heb-een-p-kluun</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theateraandeparade.nl/nl/programma/the-best-of-help-ik-heb-een-p-kluun</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I130" s="2" t="n"/>
+      <c r="J130" s="2" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C131" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-16 19:30</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr"/>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cortimedia.nl/boekestijn-en-de-wijk-live-eindejaarsshow</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="n"/>
+      <c r="J131" s="2" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C132" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-08 20:15</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr"/>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cortimedia.nl/boekestijn-en-de-wijk-live-eindejaarsshow</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="n"/>
+      <c r="J132" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6026,7 +6364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7958,6 +8296,32 @@
         <is>
           <t>Het Park</t>
         </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>De Kring (EKP-gebouw)</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Roosendaal</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Brabant</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>51.534914</v>
+      </c>
+      <c r="F65" t="n">
+        <v>4.4519129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dubbele podcast/show hersteld (Help ik heb een puber vs LIVE-variant)
- 'live' hoort er net als lidwoorden uit bij het matchen van shows,
  anders levert eenzelfde show met/zonder 'Live' in de titel een
  dubbele podcast + show + events op (dit gebeurde bij de Corti-import)
- bouw-site.py ruimt nu ook verweesde podcast-pagina's op die niet meer
  bij een bestaande podcast horen
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -583,7 +583,11 @@
         </is>
       </c>
       <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cortimedia.nl/help-ik-heb-een-puber</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Kind &amp; gezin</t>
@@ -599,7 +603,11 @@
           <t>In ruim honderd afleveringen van Help, ik heb een puber! praten schrijver Kluun en orthopedagoog Yvanka van der Zwaan met experts en met pubers zelf over opvoeden in de puberteit. In de theatershow Best of komen de meest gestelde vragen en de meest herkenbare onderwerpen uit de podcast samen in een avond met veel ruimte voor gesprek met de zaal.</t>
         </is>
       </c>
-      <c r="I4" s="2" t="n"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>1726575117</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="n"/>
     </row>
     <row r="5">
@@ -760,41 +768,6 @@
       </c>
       <c r="J8" s="2" t="n">
         <v>17</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Help, ik word volwassen!</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts221/v4/a0/1b/c4/a01bc439-71a8-107c-9d17-d667df42192b/mza_4432722255828391472.jpg/600x600bb.jpg</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://www.cortimedia.nl/help-ik-heb-een-puber</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Opvoeding</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Kluun en Yvanka van der Zwaan bespreken wekelijks de uitdagingen van het opvoeden van pubers - herkenbaar, eerlijk en met humor. De podcast heette eerder 'Help, ik heb een puber!'.</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>1726575117</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -808,7 +781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1004,31 +977,6 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Best of 'Help, ik heb een Puber'</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>theatershow</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Corti Media</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>podcast live</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1040,7 +988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1113,14 +1061,6 @@
       </c>
       <c r="B8" s="2" t="n">
         <v>7</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1134,7 +1074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J132"/>
+  <dimension ref="A1:J127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6089,24 +6029,20 @@
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B126" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C126" s="2" t="n">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 20:15</t>
-        </is>
-      </c>
-      <c r="E126" s="2" t="inlineStr">
-        <is>
-          <t>https://www.lievekamp.nl/programma/met-kluun-yvanka-van-der-zwaan-the-best-of-help-ik-heb-een-puber-07-okt-20-15/</t>
-        </is>
-      </c>
+          <t>2026-11-16 19:30</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr"/>
       <c r="F126" s="2" t="inlineStr">
         <is>
           <t>in verkoop</t>
@@ -6114,7 +6050,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>https://www.lievekamp.nl/programma/met-kluun-yvanka-van-der-zwaan-the-best-of-help-ik-heb-een-puber-07-okt-20-15/</t>
+          <t>https://www.cortimedia.nl/boekestijn-en-de-wijk-live-eindejaarsshow</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
@@ -6122,31 +6058,25 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I126" s="2" t="n">
-        <v>15</v>
-      </c>
+      <c r="I126" s="2" t="n"/>
       <c r="J126" s="2" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B127" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C127" s="2" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28 20:30</t>
-        </is>
-      </c>
-      <c r="E127" s="2" t="inlineStr">
-        <is>
-          <t>https://delamar.nl/voorstellingen/best-of-help-ik-heb-een-puber-live/</t>
-        </is>
-      </c>
+          <t>2026-12-08 20:15</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr"/>
       <c r="F127" s="2" t="inlineStr">
         <is>
           <t>in verkoop</t>
@@ -6154,7 +6084,7 @@
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>https://delamar.nl/voorstellingen/best-of-help-ik-heb-een-puber-live/</t>
+          <t>https://www.cortimedia.nl/boekestijn-en-de-wijk-live-eindejaarsshow</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr">
@@ -6162,196 +6092,8 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I127" s="2" t="n">
-        <v>19.5</v>
-      </c>
+      <c r="I127" s="2" t="n"/>
       <c r="J127" s="2" t="inlineStr"/>
-    </row>
-    <row r="128">
-      <c r="A128" s="2" t="n">
-        <v>127</v>
-      </c>
-      <c r="B128" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="C128" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="D128" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-30 20:15</t>
-        </is>
-      </c>
-      <c r="E128" s="2" t="inlineStr">
-        <is>
-          <t>https://www.spotgroningen.nl/programma/kluun-en-yvanka-van-der-zwaan/</t>
-        </is>
-      </c>
-      <c r="F128" s="2" t="inlineStr">
-        <is>
-          <t>in verkoop</t>
-        </is>
-      </c>
-      <c r="G128" s="2" t="inlineStr">
-        <is>
-          <t>https://www.spotgroningen.nl/programma/kluun-en-yvanka-van-der-zwaan/</t>
-        </is>
-      </c>
-      <c r="H128" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="I128" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="J128" s="2" t="inlineStr"/>
-    </row>
-    <row r="129">
-      <c r="A129" s="2" t="n">
-        <v>128</v>
-      </c>
-      <c r="B129" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="C129" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="D129" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-25 20:00</t>
-        </is>
-      </c>
-      <c r="E129" s="2" t="inlineStr">
-        <is>
-          <t>https://www.schouwburgconcertzaaltilburg.nl/nl/agenda/kluun-help-ik-heb-een-puber</t>
-        </is>
-      </c>
-      <c r="F129" s="2" t="inlineStr">
-        <is>
-          <t>in verkoop</t>
-        </is>
-      </c>
-      <c r="G129" s="2" t="inlineStr">
-        <is>
-          <t>https://www.schouwburgconcertzaaltilburg.nl/nl/agenda/kluun-help-ik-heb-een-puber</t>
-        </is>
-      </c>
-      <c r="H129" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="I129" s="2" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="J129" s="2" t="inlineStr"/>
-    </row>
-    <row r="130">
-      <c r="A130" s="2" t="n">
-        <v>129</v>
-      </c>
-      <c r="B130" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="C130" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="D130" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E130" s="2" t="inlineStr">
-        <is>
-          <t>https://www.theateraandeparade.nl/nl/programma/the-best-of-help-ik-heb-een-p-kluun</t>
-        </is>
-      </c>
-      <c r="F130" s="2" t="inlineStr">
-        <is>
-          <t>in verkoop</t>
-        </is>
-      </c>
-      <c r="G130" s="2" t="inlineStr">
-        <is>
-          <t>https://www.theateraandeparade.nl/nl/programma/the-best-of-help-ik-heb-een-p-kluun</t>
-        </is>
-      </c>
-      <c r="H130" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="I130" s="2" t="n"/>
-      <c r="J130" s="2" t="inlineStr"/>
-    </row>
-    <row r="131">
-      <c r="A131" s="2" t="n">
-        <v>130</v>
-      </c>
-      <c r="B131" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C131" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="D131" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-16 19:30</t>
-        </is>
-      </c>
-      <c r="E131" s="2" t="inlineStr"/>
-      <c r="F131" s="2" t="inlineStr">
-        <is>
-          <t>in verkoop</t>
-        </is>
-      </c>
-      <c r="G131" s="2" t="inlineStr">
-        <is>
-          <t>https://www.cortimedia.nl/boekestijn-en-de-wijk-live-eindejaarsshow</t>
-        </is>
-      </c>
-      <c r="H131" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="I131" s="2" t="n"/>
-      <c r="J131" s="2" t="inlineStr"/>
-    </row>
-    <row r="132">
-      <c r="A132" s="2" t="n">
-        <v>131</v>
-      </c>
-      <c r="B132" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C132" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="D132" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-08 20:15</t>
-        </is>
-      </c>
-      <c r="E132" s="2" t="inlineStr"/>
-      <c r="F132" s="2" t="inlineStr">
-        <is>
-          <t>in verkoop</t>
-        </is>
-      </c>
-      <c r="G132" s="2" t="inlineStr">
-        <is>
-          <t>https://www.cortimedia.nl/boekestijn-en-de-wijk-live-eindejaarsshow</t>
-        </is>
-      </c>
-      <c r="H132" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="I132" s="2" t="n"/>
-      <c r="J132" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
POM - Een Podcast over Media Liveshow toegevoegd (Rode Hoed, 22 sept)
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -770,6 +770,41 @@
         <v>17</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>POM - Een Podcast over Media</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts211/v4/68/d1/89/68d1893a-0636-4020-0caa-6d530d259745/mza_12575349570025535501.jpg/600x600bb.jpg</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://www.pom.show/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Media &amp; technologie</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Alexander Klopping en Ernst-Jan Pfauth bespreken wekelijks het nieuws over media, cultuur, technologie en ondernemen.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>1114136654</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -781,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -977,6 +1012,27 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Een Podcast over Media Liveshow</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>theatershow</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>podcast live</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -988,7 +1044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1061,6 +1117,14 @@
       </c>
       <c r="B8" s="2" t="n">
         <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1074,7 +1138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J127"/>
+  <dimension ref="A1:J128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6095,6 +6159,46 @@
       <c r="I127" s="2" t="n"/>
       <c r="J127" s="2" t="inlineStr"/>
     </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
+        <v>132</v>
+      </c>
+      <c r="B128" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C128" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 20:00</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>https://rodehoed.nl/programma/een-podcast-over-media-liveshow-2026/</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>https://rodehoed.nl/programma/een-podcast-over-media-liveshow-2026/</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J128" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6106,7 +6210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8064,6 +8168,32 @@
       </c>
       <c r="F65" t="n">
         <v>4.4519129</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Rode Hoed</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Holland</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>52.3773438</v>
+      </c>
+      <c r="F66" t="n">
+        <v>4.8872604</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Top-100 verder afgelopen: 8 podcasts gecheckt zonder liveshow, Alle Geschiedenis Ooit toegevoegd (13 data)
- Alle Geschiedenis Ooit - De Grote Namen Geschiedenis-show: grote tour
  gevonden via boekingskantoor friendlyfire.nl, 13 data t/m jan 2027
- Heterdaad, Vandaag Inside, KieftJansenEgmondGijp, De Jortcast,
  Moorden in de jaren, RADIO BOOS, Geschiedenis voor herbeginners,
  De Grote Podcastlas, De Nieuwe Wereld, Schuilen in Schoonheid,
  De Wit & De Wereld, Blokhuis de Podcast, Kick-off met Valentijn
  Driessen gecheckt: geen (actuele) liveshow gevonden
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -805,6 +805,39 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Alle Geschiedenis Ooit - Grote Namen</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts221/v4/94/77/71/9477713e-84ee-96d3-2574-91226f446892/mza_11947026339099286329.jpg/600x600bb.png</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Geschiedenis</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Nynke de Jong, Arco Gnocchi, Thom Aalmoes en Andrea Huntjens duiken wekelijks in de grote namen uit de geschiedenis.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>1621278264</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -816,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1033,6 +1066,31 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Alle Geschiedenis Ooit - De Grote Namen Geschiedenis-show</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>theatershow</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Friendly Fire</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>thema-verwant</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1044,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1125,6 +1183,14 @@
       </c>
       <c r="B9" s="2" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1138,7 +1204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J128"/>
+  <dimension ref="A1:J141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6199,6 +6265,510 @@
       </c>
       <c r="J128" s="2" t="inlineStr"/>
     </row>
+    <row r="129">
+      <c r="A129" s="2" t="n">
+        <v>133</v>
+      </c>
+      <c r="B129" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C129" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 20:00</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hetpostkantoor.info/event/alle-geschiedenis-ooit-de-grote-namen-geschiedenis-show</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hetpostkantoor.info/event/alle-geschiedenis-ooit-de-grote-namen-geschiedenis-show</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I129" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="J129" s="2" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n">
+        <v>134</v>
+      </c>
+      <c r="B130" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C130" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16 20:00</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kunstmin.nl/voorstellingen/alle-geschiedenis-ooit-de-grote-namen-geschiedenis-show</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kunstmin.nl/voorstellingen/alle-geschiedenis-ooit-de-grote-namen-geschiedenis-show</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I130" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="J130" s="2" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="B131" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C131" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18 14:30</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>https://www.plt.nl/programma/alle-geschiedenis-ooit/18-10-2026-14-30</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>https://www.plt.nl/programma/alle-geschiedenis-ooit/18-10-2026-14-30</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J131" s="2" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n">
+        <v>136</v>
+      </c>
+      <c r="B132" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C132" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 19:30</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kampanje.nl/voorstellingen/alle-geschiedenis-ooit-74dq</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kampanje.nl/voorstellingen/alle-geschiedenis-ooit-74dq</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="J132" s="2" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n">
+        <v>137</v>
+      </c>
+      <c r="B133" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C133" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-10 20:15</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>https://www.isalatheater.nl/agenda/alle-geschiedenis-ooit-m5zv</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>https://www.isalatheater.nl/agenda/alle-geschiedenis-ooit-m5zv</t>
+        </is>
+      </c>
+      <c r="H133" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I133" s="2" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="J133" s="2" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n">
+        <v>138</v>
+      </c>
+      <c r="B134" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C134" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-14 20:00</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>https://griffioen.vu.nl/voorstellingen/de-grote-namen-geschiedenis-show-succesoptie-alle-geschiedenis-ooit/14-11-2026-20-00</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>https://griffioen.vu.nl/voorstellingen/de-grote-namen-geschiedenis-show-succesoptie-alle-geschiedenis-ooit/14-11-2026-20-00</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="n"/>
+      <c r="J134" s="2" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n">
+        <v>139</v>
+      </c>
+      <c r="B135" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C135" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dekringroosendaal.nl/agenda/de-grote-namen-geschiedenis-show-8gmx</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dekringroosendaal.nl/agenda/de-grote-namen-geschiedenis-show-8gmx</t>
+        </is>
+      </c>
+      <c r="H135" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I135" s="2" t="n"/>
+      <c r="J135" s="2" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="B136" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C136" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-08</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>https://ontdekpoort.nl/programma/2944/alle-geschiedenis-ooit</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>https://ontdekpoort.nl/programma/2944/alle-geschiedenis-ooit</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="n"/>
+      <c r="J136" s="2" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="B137" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C137" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-11</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>https://flint.nl/agenda/alle-geschiedenis-ooit-nynke-de-jong-arco-gnocchi-thom-aalmoes-andrea-huntjens</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>https://flint.nl/agenda/alle-geschiedenis-ooit-nynke-de-jong-arco-gnocchi-thom-aalmoes-andrea-huntjens</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="n"/>
+      <c r="J137" s="2" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n">
+        <v>142</v>
+      </c>
+      <c r="B138" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C138" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-15</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theaterdeveste.nl/programma/de-grote-namen-geschiedenis-show-68vl</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theaterdeveste.nl/programma/de-grote-namen-geschiedenis-show-68vl</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="n"/>
+      <c r="J138" s="2" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n">
+        <v>143</v>
+      </c>
+      <c r="B139" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C139" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-19</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>https://leidseschouwburg-stadsgehoorzaal.nl/voorstelling/nynke-de-jong-arco-gnocchi-thom-aalmoes-en-andrea-huntjens-alle-geschiedenis-ooit</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>https://leidseschouwburg-stadsgehoorzaal.nl/voorstelling/nynke-de-jong-arco-gnocchi-thom-aalmoes-en-andrea-huntjens-alle-geschiedenis-ooit</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="n"/>
+      <c r="J139" s="2" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="B140" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C140" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>https://www.zwolsetheaters.nl/programma/2026-2027/alle-geschiedenis-ooit</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>https://www.zwolsetheaters.nl/programma/2026-2027/alle-geschiedenis-ooit</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="n"/>
+      <c r="J140" s="2" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n">
+        <v>145</v>
+      </c>
+      <c r="B141" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C141" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-26</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>https://griffioen.vu.nl/voorstellingen/de-grote-namen-geschiedenis-show-alle-geschiedenis-ooit/26-01-2027-20-00</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>https://griffioen.vu.nl/voorstellingen/de-grote-namen-geschiedenis-show-alle-geschiedenis-ooit/26-01-2027-20-00</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="n"/>
+      <c r="J141" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6210,7 +6780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8194,6 +8764,136 @@
       </c>
       <c r="F66" t="n">
         <v>4.8872604</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Het Postkantoor</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Bovenkarspel</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Holland</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>52.6977291</v>
+      </c>
+      <c r="F67" t="n">
+        <v>5.2357276</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Isala Theater</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Capelle aan den IJssel</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Zuid-Holland</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>51.9315597</v>
+      </c>
+      <c r="F68" t="n">
+        <v>4.5882206</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Griffioen</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Holland</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>52.3346074</v>
+      </c>
+      <c r="F69" t="n">
+        <v>4.8636531</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Theater Sneek / Poort</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Sneek</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Friesland</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>53.0317815</v>
+      </c>
+      <c r="F70" t="n">
+        <v>5.6562252</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Schouwburg Odeon</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Zwolle</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Overijssel</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>52.5104825</v>
+      </c>
+      <c r="F71" t="n">
+        <v>6.0918538</v>
       </c>
     </row>
   </sheetData>
@@ -8492,9 +9192,21 @@
           <t>NPO Luister / AVROTROS</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Alleen een eenmalige 'Jortcast Grand Tour' uit 2022 gevonden, niets actueels.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -8665,9 +9377,21 @@
           <t>Vandaag Inside</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>'Vandaag Inside Live' bestond (Ziggo Dome, editie t/m dec 2023), maar Ticketmaster-artiestenpagina toont nu 'geen aankomende evenementen'.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -8827,9 +9551,21 @@
           <t>Hanneke Hendrix &amp; Lotte Lentes / New Tree Media</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8873,9 +9609,21 @@
           <t>De Telegraaf</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Telegraaf true-crime podcast, geen aanwijzing voor theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -9023,9 +9771,21 @@
           <t>Leon Boelens, Max Gerritsen &amp; Hugo Noordman</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr"/>
-      <c r="G30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Eigen evenementenpagina bestaat (grotepodcastlas.nl/evenementen) met 'De Grote Podcastlas Live' in Tivoli Utrecht, maar de laatst vermelde data liggen allemaal voor vandaag - niets actueels om toe te voegen.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -9150,9 +9910,21 @@
           <t>NPO Luister / BNNVARA</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr"/>
-      <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden (wel losse 'BOOS Grote Gesprekken'-interviews, geen liveshow-format).</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -9219,9 +9991,21 @@
           <t>KieftJansenEgmondGijp</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr"/>
-      <c r="G38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden, alleen YouTube-afleveringen.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -9300,9 +10084,21 @@
           <t>Jonas Goossenaerts e.a.</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr"/>
-      <c r="F41" s="2" t="inlineStr"/>
-      <c r="G41" s="2" t="inlineStr"/>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Vlaamse podcast; 'LIVE'-reeks blijkt Kinepolis-filmavonden in Belgie, geen theatertour in Nederland.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Toplijst-tracker gecorrigeerd: 6 podcasts stonden nog niet als gecontroleerd geregistreerd (waren wel al gezocht)
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -9010,9 +9010,21 @@
           <t>Dag &amp; Nacht</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Interviewpodcast van Matthijs van Nieuwkerk (Dag en Nacht), geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -9068,9 +9080,21 @@
           <t>NPO Luister / BNNVARA</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Geopolitieke podcast van Tim de Wit en Arend Jan Boekestijn (BNNVARA/Pauw &amp; De Wit), geen aanwijzing voor een eigen theatertour gevonden (Boekestijn doet wel liveshows, maar onder Boekestijn &amp; De Wijk - zie die podcast).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -9667,9 +9691,21 @@
           <t>De Nieuwe Wereld</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -9829,9 +9865,21 @@
           <t>De Telegraaf</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Telegraaf-voetbalpodcast, geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -9852,9 +9900,21 @@
           <t>NPO Luister / BNNVARA</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr"/>
-      <c r="F33" s="2" t="inlineStr"/>
-      <c r="G33" s="2" t="inlineStr"/>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -9968,9 +10028,21 @@
           <t>Alle Geschiedenis Ooit</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr"/>
-      <c r="F37" s="2" t="inlineStr"/>
-      <c r="G37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>De Grote Namen Geschiedenis-show, 13 data gevonden via friendlyfire.nl - toegevoegd.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Top-100: 13 podcasts extra gecheckt (39 van 100 in totaal)
Universiteit van Nederland Live bleek een echte tour te zijn geweest
maar helemaal uit 2023-2024; het NPO Luister Podcastfestival (jaarlijks,
eind maart) verklaart optredens van De Dag, Verdwenen en NOS Wielerpodcast
zonder dat het een eigen tour van die podcasts is. Lessen vastgelegd in
project memory (bronnen_fase1.md).
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -9251,9 +9251,21 @@
           <t>de Volkskrant</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Dagelijkse nieuwspodcast, geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -9274,9 +9286,21 @@
           <t>NRC</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Dagelijkse nieuwspodcast, geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -9436,9 +9460,21 @@
           <t>NPO Luister / NOS</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Zelfde NPO Luister Podcastfestival als NOS Wielerpodcast (zie die notitie), verder geen eigen tour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -9494,9 +9530,21 @@
           <t>NPO Luister / EO</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Zelfde NPO Luister Podcastfestival als NOS Wielerpodcast (zie die notitie), verder geen eigen tour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -9552,9 +9600,21 @@
           <t>Dag en Nacht</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -9668,9 +9728,21 @@
           <t>NRC</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Dagelijkse nieuwspodcast, geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -10098,9 +10170,21 @@
           <t>De Telegraaf</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr"/>
-      <c r="F39" s="2" t="inlineStr"/>
-      <c r="G39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -10191,9 +10275,21 @@
           <t>Victor Vlam</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Victor Vlam deed met Lars Duursma een liveshow over De Communicado's in Veendam, maar die stond als afgelast (30 jan 2025); niets actueels.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -10237,9 +10333,21 @@
           <t>AD</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -10260,9 +10368,21 @@
           <t>NPO Luister / NOS</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr"/>
-      <c r="F45" s="2" t="inlineStr"/>
-      <c r="G45" s="2" t="inlineStr"/>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden; wel meegedaan aan het NPO Luister Podcastfestival (zie notitie NOS Wielerpodcast).</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -10333,9 +10453,21 @@
           <t>NPO Luister / NOS</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Trad op tijdens het NPO Luister Podcastfestival (21-22 maart 2026, TivoliVredenburg/Ping Pong Club Utrecht) samen met tientallen andere NPO-podcasts, maar dat is een gepasseerd tweedaags festival, geen eigen tour. Volgend jaar rond januari/februari checken of de 7e editie al data heeft.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -10379,9 +10511,21 @@
           <t>BNR Nieuwsradio</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr"/>
-      <c r="G50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Een eenmalige 'Amerika Podcast LIVE' bij Nieuwspoort bleek uit 2022, niets actueels.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -10402,9 +10546,21 @@
           <t>Teun van de Keuken &amp; Gijs Groenteman / Meer van dit</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr"/>
-      <c r="F51" s="2" t="inlineStr"/>
-      <c r="G51" s="2" t="inlineStr"/>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Gijs Groenteman deed eerder 'De Grote Harry Bannink Podcast on Tour', maar die staat als verlopen; geen actuele Teun-en-Gijs-tour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Top-100: 16 podcasts extra gecheckt (55 van 100 in totaal, geen nieuwe liveshows)
Getest op vooral true-crime en 'bekend gezicht'-genres (De Onderwereld,
Trias Criminalis, Ontvoerd naar Noord-Korea, Moordzaken, Zwijgen aan
Zee, e.a.) en boekingskantoren (Humor Werkt) - deze ronde leverde geen
nieuwe tours op, maar wel een paar bevestigingen van eenmalige/verlopen
liveshows (Echt Gebeurd bij De Parade, Moordzaken in TivoliVredenburg)
die volgend seizoen opnieuw de moeite waard zijn om te checken.
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -10403,11 +10403,19 @@
           <t>Universiteit van Nederland</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>LEAD: Universiteit van Nederland LIVE tourt, speellijst nog niet gevonden</t>
+          <t>'Universiteit van Nederland Live' bestond echt (Fuad Hassan als presentator), maar alle gevonden data zijn uit 2023-2024 en verlopen; geen actuele tour.</t>
         </is>
       </c>
     </row>
@@ -10488,9 +10496,21 @@
           <t>Jaap Jansen - Dag en Nacht Media</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr"/>
-      <c r="F49" s="2" t="inlineStr"/>
-      <c r="G49" s="2" t="inlineStr"/>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Eenmalige 'Betrouwbare Bronnen Podcast Live: Shostakovich' in het Concertgebouw was 21 september 2025 (verlopen); geen aanwijzing voor een vervolg of vaste tour.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -10581,9 +10601,21 @@
           <t>AD</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="2" t="inlineStr"/>
-      <c r="G52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -10719,9 +10751,21 @@
           <t>De Telegraaf</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr"/>
-      <c r="F58" s="2" t="inlineStr"/>
-      <c r="G58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -10742,9 +10786,21 @@
           <t>Echt Gebeurd</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr"/>
-      <c r="F59" s="2" t="inlineStr"/>
-      <c r="G59" s="2" t="inlineStr"/>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Podcastformat 'Echt Gebeurd' bracht zomer 2026 een liveversie naar De Parade (Rotterdam eind juni, Amsterdam eind juli) - inmiddels verlopen. Volgend jaar rond mei/juni checken of De Parade een nieuwe editie aankondigt.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -10765,9 +10821,21 @@
           <t>Saar Magazine</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr"/>
-      <c r="F60" s="2" t="inlineStr"/>
-      <c r="G60" s="2" t="inlineStr"/>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -10834,9 +10902,21 @@
           <t>NPO Luister / VPRO</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr"/>
-      <c r="F63" s="2" t="inlineStr"/>
-      <c r="G63" s="2" t="inlineStr"/>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Tv-interviewformat, geen theatertour; wel losse bioscoopevenementen ('op het witte doek'), dat is geen liveshow-met-publiek in de zin die wij bijhouden.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -10857,9 +10937,21 @@
           <t>Bas Dingemanse &amp; Bas van Mulken</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr"/>
-      <c r="F64" s="2" t="inlineStr"/>
-      <c r="G64" s="2" t="inlineStr"/>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -10949,9 +11041,21 @@
           <t>NPO Luister / BNNVARA</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr"/>
-      <c r="F68" s="2" t="inlineStr"/>
-      <c r="G68" s="2" t="inlineStr"/>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -10972,9 +11076,21 @@
           <t>Marian Husken, John Pel &amp; Mark Teurlings / Audiohuis</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr"/>
-      <c r="F69" s="2" t="inlineStr"/>
-      <c r="G69" s="2" t="inlineStr"/>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -11041,9 +11157,21 @@
           <t>Maxim Hartman &amp; Willem Treur</t>
         </is>
       </c>
-      <c r="E72" s="2" t="inlineStr"/>
-      <c r="F72" s="2" t="inlineStr"/>
-      <c r="G72" s="2" t="inlineStr"/>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Maxim Hartman wordt geboekt via Humor Werkt, maar geen aanwijzing voor een liveshow onder de naam van deze podcast.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -11064,9 +11192,21 @@
           <t>Tonny Media</t>
         </is>
       </c>
-      <c r="E73" s="2" t="inlineStr"/>
-      <c r="F73" s="2" t="inlineStr"/>
-      <c r="G73" s="2" t="inlineStr"/>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -11110,9 +11250,21 @@
           <t>Comedytrain</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr"/>
-      <c r="F75" s="2" t="inlineStr"/>
-      <c r="G75" s="2" t="inlineStr"/>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Podcast van Theo Maassen bij Comedytrain; geen liveshow onder de podcastnaam gevonden (Maassen doet wel eigen theatertours, maar niet als 'Ervaring voor Beginners').</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -11133,9 +11285,21 @@
           <t>Hadassah de Boer</t>
         </is>
       </c>
-      <c r="E76" s="2" t="inlineStr"/>
-      <c r="F76" s="2" t="inlineStr"/>
-      <c r="G76" s="2" t="inlineStr"/>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -11156,9 +11320,21 @@
           <t>Carrie &amp; Eddie</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr"/>
-      <c r="F77" s="2" t="inlineStr"/>
-      <c r="G77" s="2" t="inlineStr"/>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Eenmalig 'Moordzaken - De Podcast' in TivoliVredenburg was 19 december 2023 (verlopen); geen aanwijzing voor een vervolg.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -11179,9 +11355,21 @@
           <t>Grand Prix Radio</t>
         </is>
       </c>
-      <c r="E78" s="2" t="inlineStr"/>
-      <c r="F78" s="2" t="inlineStr"/>
-      <c r="G78" s="2" t="inlineStr"/>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Top-100: 13 podcasts extra gecheckt (68 van 100 in totaal)
Chantal & Tina blijft een open LEAD: &C Media noemt expliciet een
uitverkochte liveshow bij DeLaMar, maar geen bevestigde toekomstige
datum gevonden. Veldheren en Bokkenrijders bevestigd als bestaande
tours met alleen verlopen data (opnieuw checken volgend seizoen).
32 podcasts uit de top 100 staan nog open.
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -11018,9 +11018,21 @@
           <t>NPO Luister / BNNVARA</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr"/>
-      <c r="F67" s="2" t="inlineStr"/>
-      <c r="G67" s="2" t="inlineStr"/>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -11436,9 +11448,21 @@
           <t>David Lucieer, Thom Aalmoes &amp; Elisabeth Hoekstra / New Tree Media</t>
         </is>
       </c>
-      <c r="E81" s="2" t="inlineStr"/>
-      <c r="F81" s="2" t="inlineStr"/>
-      <c r="G81" s="2" t="inlineStr"/>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden (wel gemaakt door New Tree Media, dezelfde producent als Moorden in de jaren... en Rechtpraten).</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -11482,9 +11506,21 @@
           <t>AT5</t>
         </is>
       </c>
-      <c r="E83" s="2" t="inlineStr"/>
-      <c r="F83" s="2" t="inlineStr"/>
-      <c r="G83" s="2" t="inlineStr"/>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -11505,9 +11541,21 @@
           <t>Erik Scherder, Leonard Hofstra, Brechje van Bladel / Corti Media &amp; Quest</t>
         </is>
       </c>
-      <c r="E84" s="2" t="inlineStr"/>
-      <c r="F84" s="2" t="inlineStr"/>
-      <c r="G84" s="2" t="inlineStr"/>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Heeft een eigen Corti Media-pagina maar staat niet op cortimedia.nl/live; geen aanwijzing voor een theatertour.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -11528,9 +11576,21 @@
           <t>Marcel van Roosmalen, Noortje Veldhuizen &amp; Roelof de Vries</t>
         </is>
       </c>
-      <c r="E85" s="2" t="inlineStr"/>
-      <c r="F85" s="2" t="inlineStr"/>
-      <c r="G85" s="2" t="inlineStr"/>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -11574,9 +11634,21 @@
           <t>Peter van Uhm, Mart de Kruif, Jos de Groot / Corti Media</t>
         </is>
       </c>
-      <c r="E87" s="2" t="inlineStr"/>
-      <c r="F87" s="2" t="inlineStr"/>
-      <c r="G87" s="2" t="inlineStr"/>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Via Corti Media al gecheckt: 'Veldheren Live' en 'Veldheren Conferentie' bestonden echt, maar alle gevonden data (apr-jun 2025, mrt 2026) zijn verlopen.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -11597,9 +11669,21 @@
           <t>Toneelgroep Maastricht en L1</t>
         </is>
       </c>
-      <c r="E88" s="2" t="inlineStr"/>
-      <c r="F88" s="2" t="inlineStr"/>
-      <c r="G88" s="2" t="inlineStr"/>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Grote spektakelmusical van Toneelgroep Maastricht bij Stadion de Geusselt, met begeleidende podcast - maar het seizoen liep van 3 juni t/m 13 juli 2026 en is dus verlopen. Volgend jaar rond april/mei checken voor een nieuwe editie.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -11655,9 +11739,21 @@
           <t>Patrick en Eline</t>
         </is>
       </c>
-      <c r="E90" s="2" t="inlineStr"/>
-      <c r="F90" s="2" t="inlineStr"/>
-      <c r="G90" s="2" t="inlineStr"/>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -11680,7 +11776,11 @@
       </c>
       <c r="E91" s="2" t="inlineStr"/>
       <c r="F91" s="2" t="inlineStr"/>
-      <c r="G91" s="2" t="inlineStr"/>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>LEAD: &amp;C Media schrijft expliciet 'podcast, theater &amp; boek' en dat Chantal &amp; Tina hun gesprekken live op de planken brengen bij DeLaMar (inmiddels uitverkocht). Geen bevestigde toekomstige datum gevonden - TicketSwap heeft een evenement 'Aha-Erlebnissen' maar die pagina is niet op te halen. Navragen of opnieuw zoeken naar een concrete datum.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -11770,9 +11870,21 @@
           <t>AD / Tubantia</t>
         </is>
       </c>
-      <c r="E95" s="2" t="inlineStr"/>
-      <c r="F95" s="2" t="inlineStr"/>
-      <c r="G95" s="2" t="inlineStr"/>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -11793,9 +11905,21 @@
           <t>NPO Luister / PowNed</t>
         </is>
       </c>
-      <c r="E96" s="2" t="inlineStr"/>
-      <c r="F96" s="2" t="inlineStr"/>
-      <c r="G96" s="2" t="inlineStr"/>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Trad op tijdens het NPO Luister Podcastfestival (zie notitie bij NOS Wielerpodcast), geen eigen tour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -11816,9 +11940,21 @@
           <t>NPO Luister / AVROTROS</t>
         </is>
       </c>
-      <c r="E97" s="2" t="inlineStr"/>
-      <c r="F97" s="2" t="inlineStr"/>
-      <c r="G97" s="2" t="inlineStr"/>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -11839,9 +11975,21 @@
           <t>Royce de Vries &amp; Annemiek van Spanje / New Tree Media</t>
         </is>
       </c>
-      <c r="E98" s="2" t="inlineStr"/>
-      <c r="F98" s="2" t="inlineStr"/>
-      <c r="G98" s="2" t="inlineStr"/>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -11862,9 +12010,21 @@
           <t>De Correspondent</t>
         </is>
       </c>
-      <c r="E99" s="2" t="inlineStr"/>
-      <c r="F99" s="2" t="inlineStr"/>
-      <c r="G99" s="2" t="inlineStr"/>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>Heeft een sprekersagenda (decorrespondent.nl/agenda) met losse lezingen van correspondenten, maar dat is geen samenhangende show rond een specifieke podcast - valt buiten de afbakening.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Amerika in 15 minuten toegevoegd + top-100 volledig nagekeken (100/100)
- Nieuwe podcast 'Amerika in 15 minuten' met show 'De tussenstand in
  Amerika' (thema-verwant), 5 data in okt-nov 2026, gevonden via
  raymondmens.nl/theater tijdens het aflopen van de top-100.
- Twee nieuwe zalen gegeocode (Parktheater Eindhoven, Stadsschouwburg
  Utrecht).
- Toplijst-tracker afgerond: alle 100 podcasts uit de Apple top-100
  zijn nu nagekeken (was 68/100). Laatste 3 rijen ingevuld: Amerika in
  15 minuten (liveshow gevonden), De Publieke Tribune (eenmalige
  NPO-uitzending 2023, geen tour), De Brand in het Landhuis (geen
  aanwijzing gevonden).
- Site herbouwd en getest (jsdom), geen fouten.
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -838,6 +838,39 @@
         <v>36</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Amerika in 15 minuten</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts211/v4/96/92/cf/9692cfc5-8690-160a-ae98-d6dd41b4a9e4/mza_10414419130369369263.jpg/600x600bb.png</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Politiek &amp; buitenland</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Raymond Mens duidt dagelijks in 15 minuten het laatste nieuws uit de Amerikaanse politiek.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>1478135753</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -849,7 +882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1091,6 +1124,27 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>De tussenstand in Amerika</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>theatershow</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>thema-verwant</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1102,7 +1156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1191,6 +1245,14 @@
       </c>
       <c r="B10" s="2" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1204,7 +1266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J141"/>
+  <dimension ref="A1:J146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6769,6 +6831,206 @@
       <c r="I141" s="2" t="n"/>
       <c r="J141" s="2" t="inlineStr"/>
     </row>
+    <row r="142">
+      <c r="A142" s="2" t="n">
+        <v>146</v>
+      </c>
+      <c r="B142" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C142" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 21:00</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>https://www.parktheater.nl/programma/de-tussenstand-in-amerika-dh54</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>https://www.parktheater.nl/programma/de-tussenstand-in-amerika-dh54</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="J142" s="2" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n">
+        <v>147</v>
+      </c>
+      <c r="B143" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C143" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 21:00</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>https://luxortheater.nl/agenda/raymond-mens-59174</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>https://luxortheater.nl/agenda/raymond-mens-59174</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J143" s="2" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n">
+        <v>148</v>
+      </c>
+      <c r="B144" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C144" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 20:30</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>https://stadsschouwburg-utrecht.nl/agenda/de-tussenstand-in-amerika-raymond-mens</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>https://stadsschouwburg-utrecht.nl/agenda/de-tussenstand-in-amerika-raymond-mens</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="J144" s="2" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n">
+        <v>149</v>
+      </c>
+      <c r="B145" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C145" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27 21:00</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>https://www.musisenstadstheater.nl/nl/agenda/raymond-mens-de-tussenstand-in-amerika/10189</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>https://www.musisenstadstheater.nl/nl/agenda/raymond-mens-de-tussenstand-in-amerika/10189</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="J145" s="2" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="B146" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C146" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-29 14:30</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>https://delamar.nl/voorstellingen/raymond-mens/</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>https://delamar.nl/voorstellingen/raymond-mens/</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="J146" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6780,7 +7042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8894,6 +9156,58 @@
       </c>
       <c r="F71" t="n">
         <v>6.0918538</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Parktheater Eindhoven</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Eindhoven</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Brabant</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>51.4288468</v>
+      </c>
+      <c r="F72" t="n">
+        <v>5.4847037</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Stadsschouwburg Utrecht</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Utrecht</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Utrecht</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>52.0933912</v>
+      </c>
+      <c r="F73" t="n">
+        <v>5.1274954</v>
       </c>
     </row>
   </sheetData>
@@ -9356,9 +9670,21 @@
           <t>NPO Luister / EO</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -9379,9 +9705,21 @@
           <t>NPO Radio 1 / NOS</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Dagelijkse nieuwspodcast, zelfde patroon als NRC Vandaag/de Volkskrant Elke Dag - niet apart doorgezocht, geen theatertour te verwachten.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -9402,9 +9740,21 @@
           <t>Raymond Mens</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Liveshow "De tussenstand in Amerika" (thema-verwant) gevonden via raymondmens.nl/theater; 5 data toegevoegd (Eindhoven, Rotterdam, Utrecht, Arnhem, Amsterdam, okt-nov 2026). Ingeladen in de database.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -9670,9 +10020,21 @@
           <t>NPO Radio 1 / HUMAN</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Alleen een eenmalige live-uitzending gevonden: NPO Radio 1 "De Publieke Tribune - Traanjagers" op 2 sept 2023 in Theaterkerk Nes, over de walvisvaart. Geen doorlopende theatertour, geen nieuwe data gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -9798,9 +10160,21 @@
           <t>NPO Radio 1 / VPRO</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -9821,9 +10195,21 @@
           <t>Goalhanger</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Britse podcast (Goalhanger); eigen events-pagina toont alleen VK-optredens, niets in Nederland.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -9914,9 +10300,21 @@
           <t>Het Financieele Dagblad</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr"/>
-      <c r="F31" s="2" t="inlineStr"/>
-      <c r="G31" s="2" t="inlineStr"/>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Dagelijkse nieuwspodcast, zelfde patroon als NRC Vandaag/de Volkskrant Elke Dag - niet apart doorgezocht, geen theatertour te verwachten.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -10077,9 +10475,21 @@
           <t>de Volkskrant</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Interviewpodcast (Volkskrant), niet apart doorgezocht.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -10310,9 +10720,21 @@
           <t>NRC</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr"/>
-      <c r="F43" s="2" t="inlineStr"/>
-      <c r="G43" s="2" t="inlineStr"/>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Dagelijkse/wekelijkse nieuwspodcast, zelfde patroon als NRC Vandaag - niet apart doorgezocht, geen theatertour te verwachten.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -10438,9 +10860,21 @@
           <t>Alexander Klopping en Wietse Hage</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr"/>
-      <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr"/>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Nieuwspodcast over AI, niet apart doorgezocht, geen theatertour te verwachten.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -10636,9 +11070,21 @@
           <t>DPG Media</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr"/>
-      <c r="F53" s="2" t="inlineStr"/>
-      <c r="G53" s="2" t="inlineStr"/>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>'In Het Wiel: De Voorjaarsklassiekers' bestond als eenmalige theatershow in Amstelveen (mrt/apr 2024, verlopen); rond het voorjaarswielerseizoen (maart) opnieuw checken.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -10659,9 +11105,21 @@
           <t>Scientias</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr"/>
-      <c r="F54" s="2" t="inlineStr"/>
-      <c r="G54" s="2" t="inlineStr"/>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Nieuwspodcast over wetenschap, niet apart doorgezocht.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -10682,9 +11140,21 @@
           <t>Veronica Superguide</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr"/>
-      <c r="F55" s="2" t="inlineStr"/>
-      <c r="G55" s="2" t="inlineStr"/>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Nabeschouwingspodcast bij een tv-programma, niet apart doorgezocht, geen theatertour te verwachten.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -10705,9 +11175,21 @@
           <t>The Observer</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr"/>
-      <c r="F56" s="2" t="inlineStr"/>
-      <c r="G56" s="2" t="inlineStr"/>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Engelstalige podcast (The Observer), niet apart doorgezocht, geen theatertour in Nederland te verwachten.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -10728,9 +11210,21 @@
           <t>Dagblad van het Noorden</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr"/>
-      <c r="F57" s="2" t="inlineStr"/>
-      <c r="G57" s="2" t="inlineStr"/>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Regionale true-crimepodcast (Dagblad van het Noorden), niet apart doorgezocht.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -10856,9 +11350,21 @@
           <t>Universiteit van Nederland / Podimo</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr"/>
-      <c r="F61" s="2" t="inlineStr"/>
-      <c r="G61" s="2" t="inlineStr"/>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Wetenschapspodcast-spin-off, niet apart doorgezocht.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -10879,9 +11385,21 @@
           <t>Audiohuis</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr"/>
-      <c r="F62" s="2" t="inlineStr"/>
-      <c r="G62" s="2" t="inlineStr"/>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Nabeschouwingspodcast bij een tv-programma, niet apart doorgezocht, geen theatertour te verwachten.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -10972,9 +11490,21 @@
           <t>Voetbal International</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr"/>
-      <c r="F65" s="2" t="inlineStr"/>
-      <c r="G65" s="2" t="inlineStr"/>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Voetbal International-nieuwspodcast, niet apart doorgezocht, geen theatertour te verwachten.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -10995,9 +11525,21 @@
           <t>Voetbal International</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr"/>
-      <c r="F66" s="2" t="inlineStr"/>
-      <c r="G66" s="2" t="inlineStr"/>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Voetbal International-podcast, niet apart doorgezocht, geen theatertour te verwachten.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -11123,9 +11665,21 @@
           <t>NPO Radio 1 / Omroep MAX</t>
         </is>
       </c>
-      <c r="E70" s="2" t="inlineStr"/>
-      <c r="F70" s="2" t="inlineStr"/>
-      <c r="G70" s="2" t="inlineStr"/>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Nieuwsprogramma-podcast, niet apart doorgezocht, geen theatertour te verwachten.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -11146,9 +11700,21 @@
           <t>WNYC Studios &amp; OSM Audio</t>
         </is>
       </c>
-      <c r="E71" s="2" t="inlineStr"/>
-      <c r="F71" s="2" t="inlineStr"/>
-      <c r="G71" s="2" t="inlineStr"/>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Amerikaanse podcast (WNYC/OSM), geen theatertour in Nederland te verwachten.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -11239,9 +11805,21 @@
           <t>The New York Times</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr"/>
-      <c r="F74" s="2" t="inlineStr"/>
-      <c r="G74" s="2" t="inlineStr"/>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Amerikaanse podcast (The New York Times), geen theatertour in Nederland te verwachten.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -11402,9 +11980,21 @@
           <t>Dag en Nacht / Podimo</t>
         </is>
       </c>
-      <c r="E79" s="2" t="inlineStr"/>
-      <c r="F79" s="2" t="inlineStr"/>
-      <c r="G79" s="2" t="inlineStr"/>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -11425,9 +12015,21 @@
           <t>NRC</t>
         </is>
       </c>
-      <c r="E80" s="2" t="inlineStr"/>
-      <c r="F80" s="2" t="inlineStr"/>
-      <c r="G80" s="2" t="inlineStr"/>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Podcast deed eerder losse 'Onbehaarde Apen Live'-afleveringen (opgenomen voor publiek), maar geen aanwijzing voor een actuele/toekomstige datum.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -11483,9 +12085,21 @@
           <t>ESPN NL</t>
         </is>
       </c>
-      <c r="E82" s="2" t="inlineStr"/>
-      <c r="F82" s="2" t="inlineStr"/>
-      <c r="G82" s="2" t="inlineStr"/>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -11611,9 +12225,21 @@
           <t>NPO Radio 1 / VPRO</t>
         </is>
       </c>
-      <c r="E86" s="2" t="inlineStr"/>
-      <c r="F86" s="2" t="inlineStr"/>
-      <c r="G86" s="2" t="inlineStr"/>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -11774,11 +12400,19 @@
           <t>&amp;C Media / Audiohuis</t>
         </is>
       </c>
-      <c r="E91" s="2" t="inlineStr"/>
-      <c r="F91" s="2" t="inlineStr"/>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>LEAD: &amp;C Media schrijft expliciet 'podcast, theater &amp; boek' en dat Chantal &amp; Tina hun gesprekken live op de planken brengen bij DeLaMar (inmiddels uitverkocht). Geen bevestigde toekomstige datum gevonden - TicketSwap heeft een evenement 'Aha-Erlebnissen' maar die pagina is niet op te halen. Navragen of opnieuw zoeken naar een concrete datum.</t>
+          <t>Liveshow bij DeLaMar bevestigd, maar was 1 en 4 juni 2025 (verlopen); geen nieuwe datum aangekondigd.</t>
         </is>
       </c>
     </row>
@@ -11801,9 +12435,21 @@
           <t>BNR Nieuwsradio</t>
         </is>
       </c>
-      <c r="E92" s="2" t="inlineStr"/>
-      <c r="F92" s="2" t="inlineStr"/>
-      <c r="G92" s="2" t="inlineStr"/>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -11824,9 +12470,21 @@
           <t>NPO Luister / NTR</t>
         </is>
       </c>
-      <c r="E93" s="2" t="inlineStr"/>
-      <c r="F93" s="2" t="inlineStr"/>
-      <c r="G93" s="2" t="inlineStr"/>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>Gezocht op naam + theater/tickets, geen aanwijzing gevonden voor een liveshow of tour.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -11847,9 +12505,21 @@
           <t>De Telegraaf</t>
         </is>
       </c>
-      <c r="E94" s="2" t="inlineStr"/>
-      <c r="F94" s="2" t="inlineStr"/>
-      <c r="G94" s="2" t="inlineStr"/>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -12045,9 +12715,21 @@
           <t>BNR Nieuwsradio</t>
         </is>
       </c>
-      <c r="E100" s="2" t="inlineStr"/>
-      <c r="F100" s="2" t="inlineStr"/>
-      <c r="G100" s="2" t="inlineStr"/>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>Geen aanwijzing voor een theatertour gevonden.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -12068,9 +12750,21 @@
           <t>NPO Luister / VPRO</t>
         </is>
       </c>
-      <c r="E101" s="2" t="inlineStr"/>
-      <c r="F101" s="2" t="inlineStr"/>
-      <c r="G101" s="2" t="inlineStr"/>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>geen liveshow gevonden</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>'Europa Draait Door LIVE - De Verkiezingsshow' bestond echt (ITA Amsterdam, Tilburg e.a.) maar was gekoppeld aan de Europese verkiezingen van 2024 en is verlopen; pas weer relevant rond de volgende EU-verkiezingen (2029).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Producent-hubs afgelopen: De Rode Lantaarn 10 jaar toegevoegd
Dag en Nacht Media, Podimo eigen producties, NPO Luister, Spraakwater
en New Heroes gecheckt op podcast-liveshows. De meeste hubs leverden
niets nieuws op (geen tourpagina, festival-only, of geen echte
podcastproducent). Wel gevonden: De Rode Lantaarn (wielerpodcast,
Dag en Nacht Media) speelt op 27-09-2026 in TivoliVredenburg Utrecht
voor het 10-jarig bestaan van de podcast.

Onderzocht en als doodlopend genoteerd voor toekomstige sessies:
Massive Media (lijkt niet te bestaan als NL podcastproducent),
Spraakwater (is zelf een podcast, geen producent), New Heroes
(zakelijke trainingsacademie, geen podcastproducent), DAMN HONEY
theatertour (afgelopen, was najaar 2025), De Grote Podcastlas
evenementenpagina (bevat vooral pubquizzes/festivals, geen
toekomstige theatershow-datums).
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -871,6 +871,29 @@
         <v>14</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>De Rode Lantaarn</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts211/v4/6d/cb/e3/6dcbe3fb-9639-003d-18aa-a9ef930a3601/mza_2259557170486475773.jpg/600x600bb.jpg</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>1129201599</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -882,7 +905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1145,6 +1168,27 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>De Rode Lantaarn 10 jaar</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>theatershow</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>podcast live</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1156,7 +1200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1253,6 +1297,14 @@
       </c>
       <c r="B11" s="2" t="n">
         <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1266,7 +1318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J146"/>
+  <dimension ref="A1:J147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7030,6 +7082,46 @@
         <v>19.5</v>
       </c>
       <c r="J146" s="2" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n">
+        <v>151</v>
+      </c>
+      <c r="B147" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C147" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 18:30</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tivolivredenburg.nl/agenda/67853048/de-rode-lantaarn-10-jaar-27-09-2026</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tivolivredenburg.nl/agenda/67853048/de-rode-lantaarn-10-jaar-27-09-2026</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="I147" s="2" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="J147" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Banner: scherpe cover-logo + randkleuren i.p.v. vervaagde achtergrond
De banner op de podcastpagina's toont nu de cover zelf scherp (als
logo, links), met de rest van de band gevuld met de kleur(en) van de
buitenrand van die specifieke cover-afbeelding (uni waar de rand een
achtergrondkleur is, links/rechts-verloop waar de rand echt tweekleurig
is, zoals bij Boekestijn en De Wijk: zwart/geel).

Kleuren zijn per podcast bepaald door de cover in de browser op canvas
te tekenen en de dominante kleur aan de linker- en rechterrand te
bemonsteren (device_bash zelf heeft geen netwerktoegang tot de
Apple-CDN, de browser wel). Opgeslagen in twee nieuwe kolommen in het
podcasts-tabblad: bannerkleur_links en bannerkleur_rechts.
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -493,6 +493,16 @@
           <t>apple_rang</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>bannerkleur_links</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>bannerkleur_rechts</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -527,6 +537,16 @@
       </c>
       <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>#080808</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>#080808</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -567,6 +587,16 @@
       <c r="J3" s="2" t="n">
         <v>11</v>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>#983838</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>#680808</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -609,6 +639,16 @@
         </is>
       </c>
       <c r="J4" s="2" t="n"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>#e8a8a8</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>#e8b8b8</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -649,6 +689,16 @@
       <c r="J5" s="2" t="n">
         <v>3</v>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>#181818</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>#f8d808</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -689,6 +739,16 @@
       <c r="J6" s="2" t="n">
         <v>7</v>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>#f87838</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>#f87838</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -729,6 +789,16 @@
       <c r="J7" s="2" t="n">
         <v>28</v>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>#788898</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>#989898</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -769,6 +839,16 @@
       <c r="J8" s="2" t="n">
         <v>17</v>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>#a8d8c8</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>#a8d8c8</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -804,6 +884,16 @@
           <t>1114136654</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>#f87848</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>#f87848</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -837,6 +927,16 @@
       <c r="J10" s="2" t="n">
         <v>36</v>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>#3888e8</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>#3888e8</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -870,6 +970,16 @@
       <c r="J11" s="2" t="n">
         <v>14</v>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>#085888</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>#085888</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -892,6 +1002,16 @@
       </c>
       <c r="I12" t="n">
         <v>1129201599</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>#28a8e8</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>#28a8e8</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Grote theaterzalen afgespeurd: 3 nieuwe podcasts, 4 nieuwe shows
Gerichte 'podcast'-zoekopdracht op de programmering van Carre, DeLaMar,
Chasse, De Doelen, Koninklijke Schouwburg, Musis en Parktheater
(i.p.v. generieke categorie-browsing) leverde op:
- Hagelslag: extra datum bij bestaande show (De Doelen, Rotterdam)
- Culturele bagage (de Volkskrant): 'Welkom terug in het patriarchaat',
  1 toekomstige datum (Leiden, maart 2027 - eerdere data in de tour
  waren al verlopen)
- De Lesbische Liga Podcast: 'De Lesbische Liga Live' in
  TivoliVredenburg (11 sept 2026, uitverkocht)
- De Boordradio: 'De Boordradio LIVE' in Musis Arnhem (22 dec 2026)

Man man man (Koud Zweed) en Moeders of Loeders kwamen ook naar boven
maar hun tourdata bleken allemaal verlopen (2024 resp. seizoen
2025-2026); niet ingeladen, wel het signaal dat ze periodiek touren.
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1014,6 +1014,105 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Culturele bagage</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts221/v4/c2/10/d0/c210d060-0d5d-d3ca-41a8-fe287319c478/mza_7064471614632340840.jpg/600x600bb.jpg</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Media &amp; technologie</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>1616657622</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>#8898b8</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>#a8a8b8</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>De Lesbische Liga Podcast</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts211/v4/35/9c/92/359c92c3-7052-fcaf-802a-333035c7e955/mza_7283539563238062752.jpg/600x600bb.jpg</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Overig</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>1507828781</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>#f8f8f8</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>#f8f8f8</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>De Boordradio</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts211/v4/da/94/ec/da94ec1b-573b-883c-141b-dd0c06ea60dd/mza_6876213664597474478.jpg/600x600bb.jpg</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>1300085866</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>#f8f8f8</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>#f8f8f8</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1025,7 +1124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1309,6 +1408,69 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Welkom terug in het patriarchaat</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>theatershow</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>thema-verwant</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>De Lesbische Liga Live</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>theatershow</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>podcast live</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>De Boordradio LIVE</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>theatershow</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>podcast live</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1320,7 +1482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1425,6 +1587,30 @@
       </c>
       <c r="B12" s="2" t="n">
         <v>11</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1438,7 +1624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J147"/>
+  <dimension ref="A1:J151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7243,6 +7429,166 @@
       </c>
       <c r="J147" s="2" t="inlineStr"/>
     </row>
+    <row r="148">
+      <c r="A148" s="2" t="n">
+        <v>152</v>
+      </c>
+      <c r="B148" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C148" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:15</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dedoelen.nl/nl/agenda/hagelslag-de-podcast-xm31</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dedoelen.nl/nl/agenda/hagelslag-de-podcast-xm31</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="J148" s="2" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n">
+        <v>153</v>
+      </c>
+      <c r="B149" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C149" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>2027-03-02 20:15</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>https://leidseschouwburg-stadsgehoorzaal.nl/voorstelling/de-volkskrant-welkom-terug-in-het-patriarchaat-liveshow-culturele-bagage/</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>https://leidseschouwburg-stadsgehoorzaal.nl/voorstelling/de-volkskrant-welkom-terug-in-het-patriarchaat-liveshow-culturele-bagage/</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="J149" s="2" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n">
+        <v>154</v>
+      </c>
+      <c r="B150" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C150" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11 20:30</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tivolivredenburg.nl/agenda/51777282/de-lesbische-liga-live-11-09-2026</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>uitverkocht</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tivolivredenburg.nl/agenda/51777282/de-lesbische-liga-live-11-09-2026</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="I150" s="2" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="J150" s="2" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n">
+        <v>155</v>
+      </c>
+      <c r="B151" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C151" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-22 20:00</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>https://www.musisenstadstheater.nl/nl/agenda/podcast-de-boordradio-live/10193</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>https://www.musisenstadstheater.nl/nl/agenda/podcast-de-boordradio-live/10193</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="I151" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="J151" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7254,7 +7600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9420,6 +9766,32 @@
       </c>
       <c r="F73" t="n">
         <v>5.1274954</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>de Doelen</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Rotterdam</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Zuid-Holland</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>51.9220495</v>
+      </c>
+      <c r="F74" t="n">
+        <v>4.4726898</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Vul tijden en prijzen aan voor shows binnen 90 dagen
Tijd en/of prijs toegevoegd of geverifieerd voor 47 shows (Harrekidee-tour,
Boekestijn & De Wijk-tour, Over de liefde, Alle Geschiedenis Ooit), inclusief
enkele uitverkocht/wachtlijst-statussen. 5 shows missen nog alleen de prijs
(bron niet vindbaar of prijs wordt niet getoond omdat uitverkocht).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -2993,7 +2993,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I30" s="2" t="n"/>
+      <c r="I30" s="2" t="n">
+        <v>29</v>
+      </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
           <t>https://www.theaterdeveste.nl/programma/boekestijn-en-de-wijk-omarmen-de-ondergang-h9ks</t>
@@ -3144,7 +3146,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>2026-11-21</t>
+          <t>2026-11-21 20:15</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
@@ -3176,7 +3178,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>2026-11-29</t>
+          <t>2026-11-29 14:30</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -3199,7 +3201,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I35" s="2" t="n"/>
+      <c r="I35" s="2" t="n">
+        <v>23.5</v>
+      </c>
       <c r="J35" s="2" t="n"/>
     </row>
     <row r="36">
@@ -3854,7 +3858,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-19 20:15</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -3877,7 +3881,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I51" s="2" t="n"/>
+      <c r="I51" s="2" t="n">
+        <v>31</v>
+      </c>
       <c r="J51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
@@ -3892,7 +3898,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-22 20:00</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -3915,7 +3921,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I52" s="2" t="n"/>
+      <c r="I52" s="2" t="n">
+        <v>20.5</v>
+      </c>
       <c r="J52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
@@ -3970,7 +3978,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-25 20:15</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr"/>
@@ -3989,7 +3997,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I54" s="2" t="n"/>
+      <c r="I54" s="2" t="n">
+        <v>27.5</v>
+      </c>
       <c r="J54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
@@ -4054,7 +4064,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>in verkoop</t>
+          <t>uitverkocht</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -4482,7 +4492,7 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>2026-11-11</t>
+          <t>2026-11-11 20:15</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -4505,7 +4515,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I67" s="2" t="n"/>
+      <c r="I67" s="2" t="n">
+        <v>31</v>
+      </c>
       <c r="J67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
@@ -4912,7 +4924,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-09 20:00</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr"/>
@@ -4931,7 +4943,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I78" s="2" t="n"/>
+      <c r="I78" s="2" t="n">
+        <v>37.5</v>
+      </c>
       <c r="J78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
@@ -4946,7 +4960,7 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-10 20:00</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr"/>
@@ -4965,7 +4979,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I79" s="2" t="n"/>
+      <c r="I79" s="2" t="n">
+        <v>37.5</v>
+      </c>
       <c r="J79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
@@ -4980,7 +4996,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-12 20:00</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -4990,7 +5006,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>in verkoop</t>
+          <t>uitverkocht</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -5003,7 +5019,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I80" s="2" t="n"/>
+      <c r="I80" s="2" t="n">
+        <v>13.5</v>
+      </c>
       <c r="J80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
@@ -5018,7 +5036,7 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-14 20:15</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -5028,7 +5046,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>in verkoop</t>
+          <t>uitverkocht</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -5041,7 +5059,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I81" s="2" t="n"/>
+      <c r="I81" s="2" t="n">
+        <v>36</v>
+      </c>
       <c r="J81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
@@ -5056,7 +5076,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-15 20:15</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr"/>
@@ -5075,7 +5095,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I82" s="2" t="n"/>
+      <c r="I82" s="2" t="n">
+        <v>36</v>
+      </c>
       <c r="J82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
@@ -5090,7 +5112,7 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-17 20:00</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr"/>
@@ -5109,7 +5131,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I83" s="2" t="n"/>
+      <c r="I83" s="2" t="n">
+        <v>18</v>
+      </c>
       <c r="J83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
@@ -5124,7 +5148,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-21 20:00</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr"/>
@@ -5143,7 +5167,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I84" s="2" t="n"/>
+      <c r="I84" s="2" t="n">
+        <v>38</v>
+      </c>
       <c r="J84" s="2" t="inlineStr"/>
     </row>
     <row r="85">
@@ -5158,7 +5184,7 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-22 20:00</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr"/>
@@ -5177,7 +5203,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I85" s="2" t="n"/>
+      <c r="I85" s="2" t="n">
+        <v>38</v>
+      </c>
       <c r="J85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
@@ -5192,7 +5220,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-24 20:15</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr"/>
@@ -5211,7 +5239,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I86" s="2" t="n"/>
+      <c r="I86" s="2" t="n">
+        <v>36.5</v>
+      </c>
       <c r="J86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
@@ -5226,10 +5256,14 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="inlineStr"/>
+          <t>2026-09-28 20:00</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>https://www.zwolsetheaters.nl/programma/2026-2027/plien-en-bianca</t>
+        </is>
+      </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
           <t>uitverkocht</t>
@@ -5245,7 +5279,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I87" s="2" t="n"/>
+      <c r="I87" s="2" t="n">
+        <v>19</v>
+      </c>
       <c r="J87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
@@ -5260,10 +5296,14 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="E88" s="2" t="inlineStr"/>
+          <t>2026-09-29 20:00</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.zwolsetheaters.nl/programma/2026-2027/plien-en-bianca</t>
+        </is>
+      </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
           <t>uitverkocht</t>
@@ -5279,7 +5319,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I88" s="2" t="n"/>
+      <c r="I88" s="2" t="n">
+        <v>19</v>
+      </c>
       <c r="J88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
@@ -5294,7 +5336,7 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-01 20:00</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -5304,7 +5346,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>in verkoop</t>
+          <t>uitverkocht</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -5317,7 +5359,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I89" s="2" t="n"/>
+      <c r="I89" s="2" t="n">
+        <v>18</v>
+      </c>
       <c r="J89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
@@ -5332,7 +5376,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-02 20:00</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr"/>
@@ -5351,7 +5395,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I90" s="2" t="n"/>
+      <c r="I90" s="2" t="n">
+        <v>38.5</v>
+      </c>
       <c r="J90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
@@ -5366,7 +5412,7 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-05 20:00</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr"/>
@@ -5385,7 +5431,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I91" s="2" t="n"/>
+      <c r="I91" s="2" t="n">
+        <v>26.5</v>
+      </c>
       <c r="J91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
@@ -5400,7 +5448,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-06 20:00</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr"/>
@@ -5419,7 +5467,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I92" s="2" t="n"/>
+      <c r="I92" s="2" t="n">
+        <v>26.5</v>
+      </c>
       <c r="J92" s="2" t="inlineStr"/>
     </row>
     <row r="93">
@@ -5434,7 +5484,7 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-08 20:00</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr"/>
@@ -5453,7 +5503,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I93" s="2" t="n"/>
+      <c r="I93" s="2" t="n">
+        <v>35.5</v>
+      </c>
       <c r="J93" s="2" t="inlineStr"/>
     </row>
     <row r="94">
@@ -5468,7 +5520,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-19 20:15</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -5478,7 +5530,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>in verkoop</t>
+          <t>uitverkocht</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -5491,7 +5543,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I94" s="2" t="n"/>
+      <c r="I94" s="2" t="n">
+        <v>37.5</v>
+      </c>
       <c r="J94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
@@ -5506,7 +5560,7 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-20 20:00</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -5529,7 +5583,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I95" s="2" t="n"/>
+      <c r="I95" s="2" t="n">
+        <v>38.5</v>
+      </c>
       <c r="J95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
@@ -5544,7 +5600,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-22 20:15</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr"/>
@@ -5563,7 +5619,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I96" s="2" t="n"/>
+      <c r="I96" s="2" t="n">
+        <v>16</v>
+      </c>
       <c r="J96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
@@ -5578,7 +5636,7 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-26 20:15</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr"/>
@@ -5612,7 +5670,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-27 20:00</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr"/>
@@ -5631,7 +5689,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I98" s="2" t="n"/>
+      <c r="I98" s="2" t="n">
+        <v>38</v>
+      </c>
       <c r="J98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
@@ -5646,7 +5706,7 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-29 20:00</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr"/>
@@ -5665,7 +5725,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I99" s="2" t="n"/>
+      <c r="I99" s="2" t="n">
+        <v>22.25</v>
+      </c>
       <c r="J99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
@@ -5680,7 +5742,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>2026-11-02</t>
+          <t>2026-11-02 20:15</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -5703,7 +5765,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I100" s="2" t="n"/>
+      <c r="I100" s="2" t="n">
+        <v>18</v>
+      </c>
       <c r="J100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
@@ -5718,7 +5782,7 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>2026-11-03</t>
+          <t>2026-11-03 20:15</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr"/>
@@ -5737,7 +5801,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I101" s="2" t="n"/>
+      <c r="I101" s="2" t="n">
+        <v>25</v>
+      </c>
       <c r="J101" s="2" t="inlineStr"/>
     </row>
     <row r="102">
@@ -5752,10 +5818,14 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
-        </is>
-      </c>
-      <c r="E102" s="2" t="inlineStr"/>
+          <t>2026-11-05 20:00</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>https://denieuwekolk.nl/theater/agenda/plien-bianca</t>
+        </is>
+      </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
           <t>uitverkocht</t>
@@ -5771,7 +5841,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I102" s="2" t="n"/>
+      <c r="I102" s="2" t="n">
+        <v>41</v>
+      </c>
       <c r="J102" s="2" t="inlineStr"/>
     </row>
     <row r="103">
@@ -5786,7 +5858,7 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2026-11-09 20:00</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
@@ -5809,7 +5881,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I103" s="2" t="n"/>
+      <c r="I103" s="2" t="n">
+        <v>31</v>
+      </c>
       <c r="J103" s="2" t="inlineStr"/>
     </row>
     <row r="104">
@@ -5824,7 +5898,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>2026-11-10</t>
+          <t>2026-11-10 20:00</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -5847,7 +5921,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I104" s="2" t="n"/>
+      <c r="I104" s="2" t="n">
+        <v>27.5</v>
+      </c>
       <c r="J104" s="2" t="inlineStr"/>
     </row>
     <row r="105">
@@ -5862,7 +5938,7 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-11-12 20:15</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr"/>
@@ -5881,7 +5957,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I105" s="2" t="n"/>
+      <c r="I105" s="2" t="n">
+        <v>39.5</v>
+      </c>
       <c r="J105" s="2" t="inlineStr"/>
     </row>
     <row r="106">
@@ -5896,7 +5974,7 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-11-16 20:00</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr"/>
@@ -5915,7 +5993,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I106" s="2" t="n"/>
+      <c r="I106" s="2" t="n">
+        <v>38.5</v>
+      </c>
       <c r="J106" s="2" t="inlineStr"/>
     </row>
     <row r="107">
@@ -5930,7 +6010,7 @@
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>2026-11-17</t>
+          <t>2026-11-17 20:00</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr"/>
@@ -5964,7 +6044,7 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-11-19 20:15</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -5987,7 +6067,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I108" s="2" t="n"/>
+      <c r="I108" s="2" t="n">
+        <v>31.5</v>
+      </c>
       <c r="J108" s="2" t="inlineStr"/>
     </row>
     <row r="109">
@@ -6002,7 +6084,7 @@
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>2026-11-23</t>
+          <t>2026-11-23 20:00</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
@@ -6025,7 +6107,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I109" s="2" t="n"/>
+      <c r="I109" s="2" t="n">
+        <v>22</v>
+      </c>
       <c r="J109" s="2" t="inlineStr"/>
     </row>
     <row r="110">
@@ -6040,7 +6124,7 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>2026-11-24</t>
+          <t>2026-11-24 20:00</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
@@ -6063,7 +6147,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I110" s="2" t="n"/>
+      <c r="I110" s="2" t="n">
+        <v>35</v>
+      </c>
       <c r="J110" s="2" t="inlineStr"/>
     </row>
     <row r="111">
@@ -6078,7 +6164,7 @@
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>2026-11-26</t>
+          <t>2026-11-26 20:00</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
@@ -6101,7 +6187,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I111" s="2" t="n"/>
+      <c r="I111" s="2" t="n">
+        <v>28</v>
+      </c>
       <c r="J111" s="2" t="inlineStr"/>
     </row>
     <row r="112">
@@ -6116,7 +6204,7 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-30 20:15</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr"/>
@@ -6135,7 +6223,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I112" s="2" t="n"/>
+      <c r="I112" s="2" t="n">
+        <v>33</v>
+      </c>
       <c r="J112" s="2" t="inlineStr"/>
     </row>
     <row r="113">
@@ -6150,7 +6240,7 @@
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-12-01 20:00</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
@@ -6173,7 +6263,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I113" s="2" t="n"/>
+      <c r="I113" s="2" t="n">
+        <v>33</v>
+      </c>
       <c r="J113" s="2" t="inlineStr"/>
     </row>
     <row r="114">
@@ -6663,7 +6755,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I126" s="2" t="n"/>
+      <c r="I126" s="2" t="n">
+        <v>34.5</v>
+      </c>
       <c r="J126" s="2" t="inlineStr"/>
     </row>
     <row r="127">
@@ -6962,7 +7056,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>in verkoop</t>
+          <t>uitverkocht</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -6990,7 +7084,7 @@
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-30 19:30</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
@@ -7013,7 +7107,9 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="I135" s="2" t="n"/>
+      <c r="I135" s="2" t="n">
+        <v>25</v>
+      </c>
       <c r="J135" s="2" t="inlineStr"/>
     </row>
     <row r="136">

</xml_diff>

<commit_message>
Nieuwe Hagelslag-liveshow: VU Griffioen Amsterdam, 25 oktober 2026
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -1679,7 +1679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J151"/>
+  <dimension ref="A1:J152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7739,6 +7739,40 @@
         <v>26.5</v>
       </c>
       <c r="J151" s="2" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n">
+        <v>156</v>
+      </c>
+      <c r="B152" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C152" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25 15:00</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr"/>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>https://griffioen.vu.nl/</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="I152" s="2" t="n"/>
+      <c r="J152" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Voeg podcast Achter de Macht toe met 4 theatertour-data (2027)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J5CMHnCFNxEPitK1w3SQBG
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1168,6 +1168,41 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Achter de Macht</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts221/v4/b4/ba/47/b4ba474f-9299-3c69-e9ac-5752f8763c92/mza_8587266760542739759.jpeg/600x600bb.jpg</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Nieuws &amp; politiek</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Drie stemmen met elk hun eigen kijk op de Haagse politiek ontleden campagnes, peilingen en de machtsstrijd achter het nieuws.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Achter de Macht is de politieke podcast waarin oud-campagnestrateeg Bas Erlings, presentator en politicoloog Splinter Chabot en oud-Kamerlid Peter Kwint om beurten de Haagse actualiteit duiden. Ze bespreken niet alleen de inhoud van het beleid, maar vooral het spel eromheen: campagnestrategie, peilingen, coalitieonderhandelingen en de tactische zetten van politici. De aflevering verschijnt tweewekelijks en is bij luisteraars goed beoordeeld om de combinatie van insidekennis en scherpe analyse. In de theatertour lichten de makers hun podcast toe met een live show over de macht achter de macht.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>1837919848</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1179,7 +1214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1526,6 +1561,27 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Achter de Macht</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>theatershow</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>podcast live</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1537,7 +1593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1666,6 +1722,14 @@
       </c>
       <c r="B15" s="2" t="n">
         <v>14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1679,7 +1743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J152"/>
+  <dimension ref="A1:J156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7774,6 +7838,164 @@
       <c r="I152" s="2" t="n"/>
       <c r="J152" s="2" t="inlineStr"/>
     </row>
+    <row r="153">
+      <c r="A153" s="2" t="n">
+        <v>157</v>
+      </c>
+      <c r="B153" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C153" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>2027-02-09 20:00</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hnt.nl/nl/voorstellingen/achter-de-macht-djnv</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theater.nl/achter-de-macht</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="I153" s="2" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="J153" s="2" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n">
+        <v>158</v>
+      </c>
+      <c r="B154" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C154" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>2027-02-19 20:00</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>https://stadsschouwburghaarlem.nl/agenda/theatercollege-achter-de-macht</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theater.nl/achter-de-macht</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="I154" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="J154" s="2" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n">
+        <v>159</v>
+      </c>
+      <c r="B155" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C155" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>2027-03-01 20:15</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>https://cultura-ede.nl/agenda/achter-de-macht-277331/</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theater.nl/achter-de-macht</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="I155" s="2" t="n">
+        <v>27.75</v>
+      </c>
+      <c r="J155" s="2" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="B156" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C156" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>2027-03-09 20:15</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theater.nl/achter-de-macht</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theater.nl/achter-de-macht</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="I156" s="2" t="n"/>
+      <c r="J156" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7785,7 +8007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9977,6 +10199,26 @@
       </c>
       <c r="F74" t="n">
         <v>4.4726898</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Theater Cultura</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Ede</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Gelderland</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Vul coordinaten aan voor Theater Cultura (Ede)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J5CMHnCFNxEPitK1w3SQBG
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -10220,6 +10220,12 @@
           <t>Gelderland</t>
         </is>
       </c>
+      <c r="E75" t="n">
+        <v>52.0447</v>
+      </c>
+      <c r="F75" t="n">
+        <v>5.6603</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Voeg podcast Maarten van Rossem & Tom Jessen toe (theaterlezing, 21 speeldata)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J5CMHnCFNxEPitK1w3SQBG
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1203,6 +1203,44 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Maarten van Rossem &amp; Tom Jessen</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts126/v4/f5/a6/6d/f5a66dbd-6faf-86b6-f43d-2457f288e3b3/mza_5767015447653460511.jpg/600x600bb.jpg</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Nieuws &amp; politiek</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Historicus Maarten van Rossem en presentator Tom Jessen duiden wekelijks het nieuws met droge humor en historische diepgang.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Maarten van Rossem &amp; Tom Jessen is een van de best beluisterde nieuwspodcasts van Nederland. Historicus en Amerika-kenner Maarten van Rossem bespreekt samen met presentator Tom Jessen wekelijks de actualiteit, van binnenlandse politiek tot internationale verhoudingen, met zijn kenmerkende droge humor en scherpe historische duiding. Van Rossem geeft daarnaast zelfstandig theaterlezingen door het hele land, waarin hij dezelfde onderwerpen op zijn eigen manier ontleedt.</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>1513807137</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1214,7 +1252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1582,6 +1620,27 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Theaterlezing Maarten van Rossem</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>theatershow</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>zelfde makers</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1593,7 +1652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1730,6 +1789,14 @@
       </c>
       <c r="B16" s="2" t="n">
         <v>15</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -1743,7 +1810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J156"/>
+  <dimension ref="A1:J177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7996,6 +8063,814 @@
       <c r="I156" s="2" t="n"/>
       <c r="J156" s="2" t="inlineStr"/>
     </row>
+    <row r="157">
+      <c r="A157" s="2" t="n">
+        <v>161</v>
+      </c>
+      <c r="B157" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C157" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11 20:00</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G157" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H157" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I157" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="J157" s="2" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n">
+        <v>162</v>
+      </c>
+      <c r="B158" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C158" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 20:15</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G158" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H158" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I158" s="2" t="n"/>
+      <c r="J158" s="2" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n">
+        <v>163</v>
+      </c>
+      <c r="B159" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C159" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 20:00</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G159" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H159" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I159" s="2" t="n"/>
+      <c r="J159" s="2" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n">
+        <v>164</v>
+      </c>
+      <c r="B160" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C160" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02 20:30</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I160" s="2" t="n"/>
+      <c r="J160" s="2" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="n">
+        <v>165</v>
+      </c>
+      <c r="B161" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C161" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 20:00</t>
+        </is>
+      </c>
+      <c r="E161" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F161" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G161" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theater.nl/theaterlezing-maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H161" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I161" s="2" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="J161" s="2" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="n">
+        <v>166</v>
+      </c>
+      <c r="B162" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C162" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-13 20:00</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I162" s="2" t="n"/>
+      <c r="J162" s="2" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="n">
+        <v>167</v>
+      </c>
+      <c r="B163" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C163" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-20 20:00</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I163" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="J163" s="2" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="n">
+        <v>168</v>
+      </c>
+      <c r="B164" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C164" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-09 20:00</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H164" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I164" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="J164" s="2" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="n">
+        <v>169</v>
+      </c>
+      <c r="B165" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C165" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-03 15:30</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H165" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I165" s="2" t="n"/>
+      <c r="J165" s="2" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="B166" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C166" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-14 20:00</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I166" s="2" t="n"/>
+      <c r="J166" s="2" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="n">
+        <v>171</v>
+      </c>
+      <c r="B167" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C167" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-21 20:15</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H167" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I167" s="2" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="J167" s="2" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="n">
+        <v>172</v>
+      </c>
+      <c r="B168" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C168" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>2027-02-03 20:15</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I168" s="2" t="n"/>
+      <c r="J168" s="2" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="n">
+        <v>173</v>
+      </c>
+      <c r="B169" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C169" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>2027-02-12 20:00</t>
+        </is>
+      </c>
+      <c r="E169" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H169" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I169" s="2" t="n"/>
+      <c r="J169" s="2" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="n">
+        <v>174</v>
+      </c>
+      <c r="B170" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C170" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>2027-02-17 20:00</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I170" s="2" t="n"/>
+      <c r="J170" s="2" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="n">
+        <v>175</v>
+      </c>
+      <c r="B171" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C171" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>2027-03-05 20:15</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I171" s="2" t="n"/>
+      <c r="J171" s="2" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="n">
+        <v>176</v>
+      </c>
+      <c r="B172" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C172" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>2027-03-09 20:15</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I172" s="2" t="n"/>
+      <c r="J172" s="2" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n">
+        <v>177</v>
+      </c>
+      <c r="B173" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C173" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>2027-03-19 20:00</t>
+        </is>
+      </c>
+      <c r="E173" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H173" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I173" s="2" t="n"/>
+      <c r="J173" s="2" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n">
+        <v>178</v>
+      </c>
+      <c r="B174" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C174" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>2027-03-24 20:15</t>
+        </is>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I174" s="2" t="n"/>
+      <c r="J174" s="2" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="n">
+        <v>179</v>
+      </c>
+      <c r="B175" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C175" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>2027-04-15 20:00</t>
+        </is>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I175" s="2" t="n"/>
+      <c r="J175" s="2" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="B176" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C176" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>2027-05-13 20:15</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="n"/>
+      <c r="J176" s="2" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n">
+        <v>181</v>
+      </c>
+      <c r="B177" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C177" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>2027-05-20 20:15</t>
+        </is>
+      </c>
+      <c r="E177" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="inlineStr">
+        <is>
+          <t>in verkoop</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>https://www.topticketshop.nl/maarten-van-rossem</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I177" s="2" t="n"/>
+      <c r="J177" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8007,7 +8882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10225,6 +11100,396 @@
       </c>
       <c r="F75" t="n">
         <v>5.6603</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>De Oude Kerk</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Heemstede</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Holland</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>52.348</v>
+      </c>
+      <c r="F76" t="n">
+        <v>4.6155</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Dru Industrie Park</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Ulft</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Gelderland</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>51.8973</v>
+      </c>
+      <c r="F77" t="n">
+        <v>6.3898</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Theater De Omval</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Diemen</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Holland</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>52.3382</v>
+      </c>
+      <c r="F78" t="n">
+        <v>4.9592</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Ledeltheater</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Oostburg</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Zeeland</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>51.3236</v>
+      </c>
+      <c r="F79" t="n">
+        <v>3.525</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Reggehof</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Goor</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Overijssel</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>52.2506</v>
+      </c>
+      <c r="F80" t="n">
+        <v>6.5989</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Theater 't Voorhuys</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Emmeloord</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Flevoland</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>52.7103</v>
+      </c>
+      <c r="F81" t="n">
+        <v>5.748</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Theater Het Kruispunt</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Barendrecht</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Zuid-Holland</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>51.8575</v>
+      </c>
+      <c r="F82" t="n">
+        <v>4.5326</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Theater 't Speelhuis</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Helmond</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Brabant</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>51.4793</v>
+      </c>
+      <c r="F83" t="n">
+        <v>5.6567</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Geert Teis Theater</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Stadskanaal</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Groningen</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>52.9926</v>
+      </c>
+      <c r="F84" t="n">
+        <v>6.9319</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Theater De Koornbeurs</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Franeker</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Friesland</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>53.1889</v>
+      </c>
+      <c r="F85" t="n">
+        <v>5.5406</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Theater De Bussel</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Oosterhout</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Noord-Brabant</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>51.6453</v>
+      </c>
+      <c r="F86" t="n">
+        <v>4.8595</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Schaffelaartheater</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Barneveld</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>Gelderland</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>52.1425</v>
+      </c>
+      <c r="F87" t="n">
+        <v>5.5825</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Schouwburg Venray</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Venray</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Limburg</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>51.5264</v>
+      </c>
+      <c r="F88" t="n">
+        <v>5.9784</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Posthuis Theater</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Heerenveen</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>Friesland</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>52.9594</v>
+      </c>
+      <c r="F89" t="n">
+        <v>5.9181</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Theater De Storm</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Winterswijk</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Gelderland</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>51.9711</v>
+      </c>
+      <c r="F90" t="n">
+        <v>6.7189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Prijs/tijd aanvullen: Over de liefde Groningen (eerste rang nog boekbaar) en Almere (tijd + prijs)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J5CMHnCFNxEPitK1w3SQBG
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -4195,7 +4195,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>uitverkocht</t>
+          <t>in verkoop</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -4205,10 +4205,12 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="I56" s="2" t="n"/>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>29.5</v>
+      </c>
       <c r="J56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
@@ -4903,7 +4905,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>2026-12-02</t>
+          <t>2026-12-02 20:15</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -4923,10 +4925,12 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="I74" s="2" t="n"/>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>29</v>
+      </c>
       <c r="J74" s="2" t="inlineStr"/>
     </row>
     <row r="75">

</xml_diff>

<commit_message>
Prijs aanvullen: Alle Geschiedenis Ooit Griffioen Amsterdam (14 nov)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J5CMHnCFNxEPitK1w3SQBG
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -7201,10 +7201,12 @@
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="I134" s="2" t="n"/>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="n">
+        <v>27.5</v>
+      </c>
       <c r="J134" s="2" t="inlineStr"/>
     </row>
     <row r="135">

</xml_diff>

<commit_message>
Xlsx opnieuw opgeslagen (geen inhoudelijke wijziging) na bredere sourcingronde
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J5CMHnCFNxEPitK1w3SQBG
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -6735,7 +6735,7 @@
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="I122" s="2" t="n">
@@ -6851,7 +6851,7 @@
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="I125" s="2" t="n">

</xml_diff>

<commit_message>
Veroordeeld toegevoegd (speelde eerder, nu geen data)
Podcast van Lauren Fabels en strafrechtadvocaat Veerle Hammerstein (Corti Media).
Veroordeeld Live speelde in maart 2026 in de Griffioen in Amsterdam; op
cortimedia.nl/veroordeeld-live staan geen toekomstige data, dus opgenomen als
"tussen tours" net als de acht van eerder vandaag.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Va9JmdcUGDTFhKw6vFPnzJ
</commit_message>
<xml_diff>
--- a/data/podcast-liveshows.xlsx
+++ b/data/podcast-liveshows.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1722,6 +1722,66 @@
       <c r="N25" t="inlineStr">
         <is>
           <t>Chantal &amp; Tina in DeLaMar - Amsterdam, juni 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Veroordeeld</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://is1-ssl.mzstatic.com/image/thumb/Podcasts211/v4/31/b0/bb/31b0bbdc-30eb-fb1c-ccac-76805ea806bd/mza_2487447630942247232.jpg/600x600bb.png</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://www.cortimedia.nl/veroordeeld</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>True crime</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Lauren Fabels en strafrechtadvocaat Veerle Hammerstein praten met mensen die veroordeeld zijn, over hoe het zover kwam en wat dat stempel met je doet.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>In Veroordeeld gaan podcastmaker Lauren Fabels en strafrechtadvocaat Veerle Hammerstein in gesprek met mensen die voor een misdrijf zijn veroordeeld. Niet over de zaak zoals die in de krant stond, maar over het eerlijke verhaal erachter: hoe iemand tot die keuze kwam, wat er aan voorafging, en hoe het is om daarna verder te leven met een etiket dat niet meer weggaat. Dat levert gesprekken op die ongemakkelijker en menselijker zijn dan de meeste true crime. De liveversie speelde in maart 2026 in de Griffioen in Amsterdam.</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>1746090802</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>#aa9a89</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>#aa9a89</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>tussen tours</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Veroordeeld Live - Griffioen Amsterdam, maart 2026</t>
         </is>
       </c>
     </row>

</xml_diff>